<commit_message>
feat(space): simplify corridor opening and enable jumping
</commit_message>
<xml_diff>
--- a/docs/assets/space-exhibit-index.xlsx
+++ b/docs/assets/space-exhibit-index.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="education" sheetId="1" r:id="R3840e5ff38ea4d72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="professional_practice" sheetId="2" r:id="R3776614819d54ebc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="personal_archive" sheetId="3" r:id="R68da785e4d8047b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="explore" sheetId="4" r:id="R1574d6a536c8426d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="education" sheetId="1" r:id="R068516fa9ac04fad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="professional_practice" sheetId="2" r:id="R2207edc4af454bbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="personal_archive" sheetId="3" r:id="R0c4b1f37ad7044e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="explore" sheetId="4" r:id="R22d8fc92f72a4073"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9949,109 +9949,93 @@
       <x:c r="CR29" t="str"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" t="str">
-        <x:v>ui_copy</x:v>
-      </x:c>
-      <x:c r="B30" t="str">
-        <x:v>i18n_space_guide</x:v>
-      </x:c>
-      <x:c r="C30" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="D30" t="str">
-        <x:v>3009</x:v>
-      </x:c>
-      <x:c r="E30" t="str"/>
-      <x:c r="F30" t="str"/>
-      <x:c r="G30" t="str"/>
-      <x:c r="H30" t="str"/>
-      <x:c r="I30" t="str"/>
-      <x:c r="J30" t="str"/>
-      <x:c r="K30" t="str"/>
-      <x:c r="L30" t="str"/>
-      <x:c r="M30" t="str"/>
-      <x:c r="N30" t="str"/>
-      <x:c r="O30" t="str"/>
-      <x:c r="P30" t="str"/>
-      <x:c r="Q30" t="str"/>
-      <x:c r="R30" t="str"/>
-      <x:c r="S30" t="str"/>
-      <x:c r="T30" t="str"/>
-      <x:c r="U30" t="str"/>
-      <x:c r="V30" t="str"/>
-      <x:c r="W30" t="str"/>
-      <x:c r="X30" t="str"/>
-      <x:c r="Y30" t="str"/>
-      <x:c r="Z30" t="str"/>
-      <x:c r="AA30" t="str"/>
-      <x:c r="AB30" t="str"/>
-      <x:c r="AC30" t="str"/>
-      <x:c r="AD30" t="str"/>
-      <x:c r="AE30" t="str"/>
-      <x:c r="AF30" t="str"/>
-      <x:c r="AG30" t="str"/>
-      <x:c r="AH30" t="str"/>
-      <x:c r="AI30" t="str"/>
-      <x:c r="AJ30" t="str"/>
-      <x:c r="AK30" t="str"/>
-      <x:c r="AL30" t="str"/>
-      <x:c r="AM30" t="str"/>
-      <x:c r="AN30" t="str"/>
-      <x:c r="AO30" t="str"/>
-      <x:c r="AP30" t="str"/>
-      <x:c r="AQ30" t="str"/>
-      <x:c r="AR30" t="str"/>
-      <x:c r="AS30" t="str"/>
-      <x:c r="AT30" t="str"/>
-      <x:c r="AU30" t="str"/>
-      <x:c r="AV30" t="str"/>
-      <x:c r="AW30" t="str"/>
-      <x:c r="AX30" t="str"/>
-      <x:c r="AY30" t="str"/>
-      <x:c r="AZ30" t="str"/>
-      <x:c r="BA30" t="str"/>
-      <x:c r="BB30" t="str"/>
-      <x:c r="BC30" t="str"/>
-      <x:c r="BD30" t="str"/>
-      <x:c r="BE30" t="str"/>
-      <x:c r="BF30" t="str"/>
-      <x:c r="BG30" t="str"/>
-      <x:c r="BH30" t="str"/>
-      <x:c r="BI30" t="str"/>
-      <x:c r="BJ30" t="str"/>
-      <x:c r="BK30" t="str"/>
-      <x:c r="BL30" t="str"/>
-      <x:c r="BM30" t="str"/>
-      <x:c r="BN30" t="str"/>
-      <x:c r="BO30" t="str"/>
-      <x:c r="BP30" t="str"/>
-      <x:c r="BQ30" t="str"/>
-      <x:c r="BR30" t="str"/>
-      <x:c r="BS30" t="str"/>
-      <x:c r="BT30" t="str"/>
-      <x:c r="BU30" t="str"/>
-      <x:c r="BV30" t="str"/>
-      <x:c r="BW30" t="str"/>
-      <x:c r="BX30" t="str"/>
-      <x:c r="BY30" t="str"/>
-      <x:c r="BZ30" t="str"/>
-      <x:c r="CA30" t="str"/>
-      <x:c r="CB30" t="str"/>
-      <x:c r="CC30" t="str"/>
-      <x:c r="CD30" t="str"/>
-      <x:c r="CE30" t="str"/>
-      <x:c r="CF30" t="str">
-        <x:v>i18n</x:v>
-      </x:c>
-      <x:c r="CG30" t="str">
-        <x:v>space.guide</x:v>
-      </x:c>
-      <x:c r="CH30" t="str">
-        <x:v>WASD to move · Mouse to look · Aim at an exhibit, then click</x:v>
-      </x:c>
-      <x:c r="CI30" t="str">
-        <x:v>WASD 漫游 · 鼠标环顾 · 准星对准展品后点击</x:v>
-      </x:c>
+      <x:c r="A30"/>
+      <x:c r="B30"/>
+      <x:c r="C30"/>
+      <x:c r="D30"/>
+      <x:c r="E30"/>
+      <x:c r="F30"/>
+      <x:c r="G30"/>
+      <x:c r="H30"/>
+      <x:c r="I30"/>
+      <x:c r="J30"/>
+      <x:c r="K30"/>
+      <x:c r="L30"/>
+      <x:c r="M30"/>
+      <x:c r="N30"/>
+      <x:c r="O30"/>
+      <x:c r="P30"/>
+      <x:c r="Q30"/>
+      <x:c r="R30"/>
+      <x:c r="S30"/>
+      <x:c r="T30"/>
+      <x:c r="U30"/>
+      <x:c r="V30"/>
+      <x:c r="W30"/>
+      <x:c r="X30"/>
+      <x:c r="Y30"/>
+      <x:c r="Z30"/>
+      <x:c r="AA30"/>
+      <x:c r="AB30"/>
+      <x:c r="AC30"/>
+      <x:c r="AD30"/>
+      <x:c r="AE30"/>
+      <x:c r="AF30"/>
+      <x:c r="AG30"/>
+      <x:c r="AH30"/>
+      <x:c r="AI30"/>
+      <x:c r="AJ30"/>
+      <x:c r="AK30"/>
+      <x:c r="AL30"/>
+      <x:c r="AM30"/>
+      <x:c r="AN30"/>
+      <x:c r="AO30"/>
+      <x:c r="AP30"/>
+      <x:c r="AQ30"/>
+      <x:c r="AR30"/>
+      <x:c r="AS30"/>
+      <x:c r="AT30"/>
+      <x:c r="AU30"/>
+      <x:c r="AV30"/>
+      <x:c r="AW30"/>
+      <x:c r="AX30"/>
+      <x:c r="AY30"/>
+      <x:c r="AZ30"/>
+      <x:c r="BA30"/>
+      <x:c r="BB30"/>
+      <x:c r="BC30"/>
+      <x:c r="BD30"/>
+      <x:c r="BE30"/>
+      <x:c r="BF30"/>
+      <x:c r="BG30"/>
+      <x:c r="BH30"/>
+      <x:c r="BI30"/>
+      <x:c r="BJ30"/>
+      <x:c r="BK30"/>
+      <x:c r="BL30"/>
+      <x:c r="BM30"/>
+      <x:c r="BN30"/>
+      <x:c r="BO30"/>
+      <x:c r="BP30"/>
+      <x:c r="BQ30"/>
+      <x:c r="BR30"/>
+      <x:c r="BS30"/>
+      <x:c r="BT30"/>
+      <x:c r="BU30"/>
+      <x:c r="BV30"/>
+      <x:c r="BW30"/>
+      <x:c r="BX30"/>
+      <x:c r="BY30"/>
+      <x:c r="BZ30"/>
+      <x:c r="CA30"/>
+      <x:c r="CB30"/>
+      <x:c r="CC30"/>
+      <x:c r="CD30"/>
+      <x:c r="CE30"/>
+      <x:c r="CF30"/>
+      <x:c r="CG30"/>
+      <x:c r="CH30"/>
+      <x:c r="CI30"/>
       <x:c r="CJ30" t="str"/>
       <x:c r="CK30" t="str"/>
       <x:c r="CL30" t="str"/>
@@ -10975,109 +10959,93 @@
       <x:c r="CR38" t="str"/>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" t="str">
-        <x:v>ui_copy</x:v>
-      </x:c>
-      <x:c r="B39" t="str">
-        <x:v>i18n_space_jumpQuiet</x:v>
-      </x:c>
-      <x:c r="C39" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="D39" t="str">
-        <x:v>3018</x:v>
-      </x:c>
-      <x:c r="E39" t="str"/>
-      <x:c r="F39" t="str"/>
-      <x:c r="G39" t="str"/>
-      <x:c r="H39" t="str"/>
-      <x:c r="I39" t="str"/>
-      <x:c r="J39" t="str"/>
-      <x:c r="K39" t="str"/>
-      <x:c r="L39" t="str"/>
-      <x:c r="M39" t="str"/>
-      <x:c r="N39" t="str"/>
-      <x:c r="O39" t="str"/>
-      <x:c r="P39" t="str"/>
-      <x:c r="Q39" t="str"/>
-      <x:c r="R39" t="str"/>
-      <x:c r="S39" t="str"/>
-      <x:c r="T39" t="str"/>
-      <x:c r="U39" t="str"/>
-      <x:c r="V39" t="str"/>
-      <x:c r="W39" t="str"/>
-      <x:c r="X39" t="str"/>
-      <x:c r="Y39" t="str"/>
-      <x:c r="Z39" t="str"/>
-      <x:c r="AA39" t="str"/>
-      <x:c r="AB39" t="str"/>
-      <x:c r="AC39" t="str"/>
-      <x:c r="AD39" t="str"/>
-      <x:c r="AE39" t="str"/>
-      <x:c r="AF39" t="str"/>
-      <x:c r="AG39" t="str"/>
-      <x:c r="AH39" t="str"/>
-      <x:c r="AI39" t="str"/>
-      <x:c r="AJ39" t="str"/>
-      <x:c r="AK39" t="str"/>
-      <x:c r="AL39" t="str"/>
-      <x:c r="AM39" t="str"/>
-      <x:c r="AN39" t="str"/>
-      <x:c r="AO39" t="str"/>
-      <x:c r="AP39" t="str"/>
-      <x:c r="AQ39" t="str"/>
-      <x:c r="AR39" t="str"/>
-      <x:c r="AS39" t="str"/>
-      <x:c r="AT39" t="str"/>
-      <x:c r="AU39" t="str"/>
-      <x:c r="AV39" t="str"/>
-      <x:c r="AW39" t="str"/>
-      <x:c r="AX39" t="str"/>
-      <x:c r="AY39" t="str"/>
-      <x:c r="AZ39" t="str"/>
-      <x:c r="BA39" t="str"/>
-      <x:c r="BB39" t="str"/>
-      <x:c r="BC39" t="str"/>
-      <x:c r="BD39" t="str"/>
-      <x:c r="BE39" t="str"/>
-      <x:c r="BF39" t="str"/>
-      <x:c r="BG39" t="str"/>
-      <x:c r="BH39" t="str"/>
-      <x:c r="BI39" t="str"/>
-      <x:c r="BJ39" t="str"/>
-      <x:c r="BK39" t="str"/>
-      <x:c r="BL39" t="str"/>
-      <x:c r="BM39" t="str"/>
-      <x:c r="BN39" t="str"/>
-      <x:c r="BO39" t="str"/>
-      <x:c r="BP39" t="str"/>
-      <x:c r="BQ39" t="str"/>
-      <x:c r="BR39" t="str"/>
-      <x:c r="BS39" t="str"/>
-      <x:c r="BT39" t="str"/>
-      <x:c r="BU39" t="str"/>
-      <x:c r="BV39" t="str"/>
-      <x:c r="BW39" t="str"/>
-      <x:c r="BX39" t="str"/>
-      <x:c r="BY39" t="str"/>
-      <x:c r="BZ39" t="str"/>
-      <x:c r="CA39" t="str"/>
-      <x:c r="CB39" t="str"/>
-      <x:c r="CC39" t="str"/>
-      <x:c r="CD39" t="str"/>
-      <x:c r="CE39" t="str"/>
-      <x:c r="CF39" t="str">
-        <x:v>i18n</x:v>
-      </x:c>
-      <x:c r="CG39" t="str">
-        <x:v>space.jumpQuiet</x:v>
-      </x:c>
-      <x:c r="CH39" t="str">
-        <x:v>Quiet in the gallery. No jumping yet.</x:v>
-      </x:c>
-      <x:c r="CI39" t="str">
-        <x:v>在展厅要保持安静，不允许跳跃</x:v>
-      </x:c>
+      <x:c r="A39"/>
+      <x:c r="B39"/>
+      <x:c r="C39"/>
+      <x:c r="D39"/>
+      <x:c r="E39"/>
+      <x:c r="F39"/>
+      <x:c r="G39"/>
+      <x:c r="H39"/>
+      <x:c r="I39"/>
+      <x:c r="J39"/>
+      <x:c r="K39"/>
+      <x:c r="L39"/>
+      <x:c r="M39"/>
+      <x:c r="N39"/>
+      <x:c r="O39"/>
+      <x:c r="P39"/>
+      <x:c r="Q39"/>
+      <x:c r="R39"/>
+      <x:c r="S39"/>
+      <x:c r="T39"/>
+      <x:c r="U39"/>
+      <x:c r="V39"/>
+      <x:c r="W39"/>
+      <x:c r="X39"/>
+      <x:c r="Y39"/>
+      <x:c r="Z39"/>
+      <x:c r="AA39"/>
+      <x:c r="AB39"/>
+      <x:c r="AC39"/>
+      <x:c r="AD39"/>
+      <x:c r="AE39"/>
+      <x:c r="AF39"/>
+      <x:c r="AG39"/>
+      <x:c r="AH39"/>
+      <x:c r="AI39"/>
+      <x:c r="AJ39"/>
+      <x:c r="AK39"/>
+      <x:c r="AL39"/>
+      <x:c r="AM39"/>
+      <x:c r="AN39"/>
+      <x:c r="AO39"/>
+      <x:c r="AP39"/>
+      <x:c r="AQ39"/>
+      <x:c r="AR39"/>
+      <x:c r="AS39"/>
+      <x:c r="AT39"/>
+      <x:c r="AU39"/>
+      <x:c r="AV39"/>
+      <x:c r="AW39"/>
+      <x:c r="AX39"/>
+      <x:c r="AY39"/>
+      <x:c r="AZ39"/>
+      <x:c r="BA39"/>
+      <x:c r="BB39"/>
+      <x:c r="BC39"/>
+      <x:c r="BD39"/>
+      <x:c r="BE39"/>
+      <x:c r="BF39"/>
+      <x:c r="BG39"/>
+      <x:c r="BH39"/>
+      <x:c r="BI39"/>
+      <x:c r="BJ39"/>
+      <x:c r="BK39"/>
+      <x:c r="BL39"/>
+      <x:c r="BM39"/>
+      <x:c r="BN39"/>
+      <x:c r="BO39"/>
+      <x:c r="BP39"/>
+      <x:c r="BQ39"/>
+      <x:c r="BR39"/>
+      <x:c r="BS39"/>
+      <x:c r="BT39"/>
+      <x:c r="BU39"/>
+      <x:c r="BV39"/>
+      <x:c r="BW39"/>
+      <x:c r="BX39"/>
+      <x:c r="BY39"/>
+      <x:c r="BZ39"/>
+      <x:c r="CA39"/>
+      <x:c r="CB39"/>
+      <x:c r="CC39"/>
+      <x:c r="CD39"/>
+      <x:c r="CE39"/>
+      <x:c r="CF39"/>
+      <x:c r="CG39"/>
+      <x:c r="CH39"/>
+      <x:c r="CI39"/>
       <x:c r="CJ39" t="str"/>
       <x:c r="CK39" t="str"/>
       <x:c r="CL39" t="str"/>
@@ -11089,109 +11057,93 @@
       <x:c r="CR39" t="str"/>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" t="str">
-        <x:v>ui_copy</x:v>
-      </x:c>
-      <x:c r="B40" t="str">
-        <x:v>i18n_space_jumpUnlocked</x:v>
-      </x:c>
-      <x:c r="C40" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="D40" t="str">
-        <x:v>3019</x:v>
-      </x:c>
-      <x:c r="E40" t="str"/>
-      <x:c r="F40" t="str"/>
-      <x:c r="G40" t="str"/>
-      <x:c r="H40" t="str"/>
-      <x:c r="I40" t="str"/>
-      <x:c r="J40" t="str"/>
-      <x:c r="K40" t="str"/>
-      <x:c r="L40" t="str"/>
-      <x:c r="M40" t="str"/>
-      <x:c r="N40" t="str"/>
-      <x:c r="O40" t="str"/>
-      <x:c r="P40" t="str"/>
-      <x:c r="Q40" t="str"/>
-      <x:c r="R40" t="str"/>
-      <x:c r="S40" t="str"/>
-      <x:c r="T40" t="str"/>
-      <x:c r="U40" t="str"/>
-      <x:c r="V40" t="str"/>
-      <x:c r="W40" t="str"/>
-      <x:c r="X40" t="str"/>
-      <x:c r="Y40" t="str"/>
-      <x:c r="Z40" t="str"/>
-      <x:c r="AA40" t="str"/>
-      <x:c r="AB40" t="str"/>
-      <x:c r="AC40" t="str"/>
-      <x:c r="AD40" t="str"/>
-      <x:c r="AE40" t="str"/>
-      <x:c r="AF40" t="str"/>
-      <x:c r="AG40" t="str"/>
-      <x:c r="AH40" t="str"/>
-      <x:c r="AI40" t="str"/>
-      <x:c r="AJ40" t="str"/>
-      <x:c r="AK40" t="str"/>
-      <x:c r="AL40" t="str"/>
-      <x:c r="AM40" t="str"/>
-      <x:c r="AN40" t="str"/>
-      <x:c r="AO40" t="str"/>
-      <x:c r="AP40" t="str"/>
-      <x:c r="AQ40" t="str"/>
-      <x:c r="AR40" t="str"/>
-      <x:c r="AS40" t="str"/>
-      <x:c r="AT40" t="str"/>
-      <x:c r="AU40" t="str"/>
-      <x:c r="AV40" t="str"/>
-      <x:c r="AW40" t="str"/>
-      <x:c r="AX40" t="str"/>
-      <x:c r="AY40" t="str"/>
-      <x:c r="AZ40" t="str"/>
-      <x:c r="BA40" t="str"/>
-      <x:c r="BB40" t="str"/>
-      <x:c r="BC40" t="str"/>
-      <x:c r="BD40" t="str"/>
-      <x:c r="BE40" t="str"/>
-      <x:c r="BF40" t="str"/>
-      <x:c r="BG40" t="str"/>
-      <x:c r="BH40" t="str"/>
-      <x:c r="BI40" t="str"/>
-      <x:c r="BJ40" t="str"/>
-      <x:c r="BK40" t="str"/>
-      <x:c r="BL40" t="str"/>
-      <x:c r="BM40" t="str"/>
-      <x:c r="BN40" t="str"/>
-      <x:c r="BO40" t="str"/>
-      <x:c r="BP40" t="str"/>
-      <x:c r="BQ40" t="str"/>
-      <x:c r="BR40" t="str"/>
-      <x:c r="BS40" t="str"/>
-      <x:c r="BT40" t="str"/>
-      <x:c r="BU40" t="str"/>
-      <x:c r="BV40" t="str"/>
-      <x:c r="BW40" t="str"/>
-      <x:c r="BX40" t="str"/>
-      <x:c r="BY40" t="str"/>
-      <x:c r="BZ40" t="str"/>
-      <x:c r="CA40" t="str"/>
-      <x:c r="CB40" t="str"/>
-      <x:c r="CC40" t="str"/>
-      <x:c r="CD40" t="str"/>
-      <x:c r="CE40" t="str"/>
-      <x:c r="CF40" t="str">
-        <x:v>i18n</x:v>
-      </x:c>
-      <x:c r="CG40" t="str">
-        <x:v>space.jumpUnlocked</x:v>
-      </x:c>
-      <x:c r="CH40" t="str">
-        <x:v>Fine, you win.</x:v>
-      </x:c>
-      <x:c r="CI40" t="str">
-        <x:v>真拿你没办法～</x:v>
-      </x:c>
+      <x:c r="A40"/>
+      <x:c r="B40"/>
+      <x:c r="C40"/>
+      <x:c r="D40"/>
+      <x:c r="E40"/>
+      <x:c r="F40"/>
+      <x:c r="G40"/>
+      <x:c r="H40"/>
+      <x:c r="I40"/>
+      <x:c r="J40"/>
+      <x:c r="K40"/>
+      <x:c r="L40"/>
+      <x:c r="M40"/>
+      <x:c r="N40"/>
+      <x:c r="O40"/>
+      <x:c r="P40"/>
+      <x:c r="Q40"/>
+      <x:c r="R40"/>
+      <x:c r="S40"/>
+      <x:c r="T40"/>
+      <x:c r="U40"/>
+      <x:c r="V40"/>
+      <x:c r="W40"/>
+      <x:c r="X40"/>
+      <x:c r="Y40"/>
+      <x:c r="Z40"/>
+      <x:c r="AA40"/>
+      <x:c r="AB40"/>
+      <x:c r="AC40"/>
+      <x:c r="AD40"/>
+      <x:c r="AE40"/>
+      <x:c r="AF40"/>
+      <x:c r="AG40"/>
+      <x:c r="AH40"/>
+      <x:c r="AI40"/>
+      <x:c r="AJ40"/>
+      <x:c r="AK40"/>
+      <x:c r="AL40"/>
+      <x:c r="AM40"/>
+      <x:c r="AN40"/>
+      <x:c r="AO40"/>
+      <x:c r="AP40"/>
+      <x:c r="AQ40"/>
+      <x:c r="AR40"/>
+      <x:c r="AS40"/>
+      <x:c r="AT40"/>
+      <x:c r="AU40"/>
+      <x:c r="AV40"/>
+      <x:c r="AW40"/>
+      <x:c r="AX40"/>
+      <x:c r="AY40"/>
+      <x:c r="AZ40"/>
+      <x:c r="BA40"/>
+      <x:c r="BB40"/>
+      <x:c r="BC40"/>
+      <x:c r="BD40"/>
+      <x:c r="BE40"/>
+      <x:c r="BF40"/>
+      <x:c r="BG40"/>
+      <x:c r="BH40"/>
+      <x:c r="BI40"/>
+      <x:c r="BJ40"/>
+      <x:c r="BK40"/>
+      <x:c r="BL40"/>
+      <x:c r="BM40"/>
+      <x:c r="BN40"/>
+      <x:c r="BO40"/>
+      <x:c r="BP40"/>
+      <x:c r="BQ40"/>
+      <x:c r="BR40"/>
+      <x:c r="BS40"/>
+      <x:c r="BT40"/>
+      <x:c r="BU40"/>
+      <x:c r="BV40"/>
+      <x:c r="BW40"/>
+      <x:c r="BX40"/>
+      <x:c r="BY40"/>
+      <x:c r="BZ40"/>
+      <x:c r="CA40"/>
+      <x:c r="CB40"/>
+      <x:c r="CC40"/>
+      <x:c r="CD40"/>
+      <x:c r="CE40"/>
+      <x:c r="CF40"/>
+      <x:c r="CG40"/>
+      <x:c r="CH40"/>
+      <x:c r="CI40"/>
       <x:c r="CJ40" t="str"/>
       <x:c r="CK40" t="str"/>
       <x:c r="CL40" t="str"/>
@@ -11203,109 +11155,93 @@
       <x:c r="CR40" t="str"/>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" t="str">
-        <x:v>ui_copy</x:v>
-      </x:c>
-      <x:c r="B41" t="str">
-        <x:v>i18n_space_onboarding_notice</x:v>
-      </x:c>
-      <x:c r="C41" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="D41" t="str">
-        <x:v>3020</x:v>
-      </x:c>
-      <x:c r="E41" t="str"/>
-      <x:c r="F41" t="str"/>
-      <x:c r="G41" t="str"/>
-      <x:c r="H41" t="str"/>
-      <x:c r="I41" t="str"/>
-      <x:c r="J41" t="str"/>
-      <x:c r="K41" t="str"/>
-      <x:c r="L41" t="str"/>
-      <x:c r="M41" t="str"/>
-      <x:c r="N41" t="str"/>
-      <x:c r="O41" t="str"/>
-      <x:c r="P41" t="str"/>
-      <x:c r="Q41" t="str"/>
-      <x:c r="R41" t="str"/>
-      <x:c r="S41" t="str"/>
-      <x:c r="T41" t="str"/>
-      <x:c r="U41" t="str"/>
-      <x:c r="V41" t="str"/>
-      <x:c r="W41" t="str"/>
-      <x:c r="X41" t="str"/>
-      <x:c r="Y41" t="str"/>
-      <x:c r="Z41" t="str"/>
-      <x:c r="AA41" t="str"/>
-      <x:c r="AB41" t="str"/>
-      <x:c r="AC41" t="str"/>
-      <x:c r="AD41" t="str"/>
-      <x:c r="AE41" t="str"/>
-      <x:c r="AF41" t="str"/>
-      <x:c r="AG41" t="str"/>
-      <x:c r="AH41" t="str"/>
-      <x:c r="AI41" t="str"/>
-      <x:c r="AJ41" t="str"/>
-      <x:c r="AK41" t="str"/>
-      <x:c r="AL41" t="str"/>
-      <x:c r="AM41" t="str"/>
-      <x:c r="AN41" t="str"/>
-      <x:c r="AO41" t="str"/>
-      <x:c r="AP41" t="str"/>
-      <x:c r="AQ41" t="str"/>
-      <x:c r="AR41" t="str"/>
-      <x:c r="AS41" t="str"/>
-      <x:c r="AT41" t="str"/>
-      <x:c r="AU41" t="str"/>
-      <x:c r="AV41" t="str"/>
-      <x:c r="AW41" t="str"/>
-      <x:c r="AX41" t="str"/>
-      <x:c r="AY41" t="str"/>
-      <x:c r="AZ41" t="str"/>
-      <x:c r="BA41" t="str"/>
-      <x:c r="BB41" t="str"/>
-      <x:c r="BC41" t="str"/>
-      <x:c r="BD41" t="str"/>
-      <x:c r="BE41" t="str"/>
-      <x:c r="BF41" t="str"/>
-      <x:c r="BG41" t="str"/>
-      <x:c r="BH41" t="str"/>
-      <x:c r="BI41" t="str"/>
-      <x:c r="BJ41" t="str"/>
-      <x:c r="BK41" t="str"/>
-      <x:c r="BL41" t="str"/>
-      <x:c r="BM41" t="str"/>
-      <x:c r="BN41" t="str"/>
-      <x:c r="BO41" t="str"/>
-      <x:c r="BP41" t="str"/>
-      <x:c r="BQ41" t="str"/>
-      <x:c r="BR41" t="str"/>
-      <x:c r="BS41" t="str"/>
-      <x:c r="BT41" t="str"/>
-      <x:c r="BU41" t="str"/>
-      <x:c r="BV41" t="str"/>
-      <x:c r="BW41" t="str"/>
-      <x:c r="BX41" t="str"/>
-      <x:c r="BY41" t="str"/>
-      <x:c r="BZ41" t="str"/>
-      <x:c r="CA41" t="str"/>
-      <x:c r="CB41" t="str"/>
-      <x:c r="CC41" t="str"/>
-      <x:c r="CD41" t="str"/>
-      <x:c r="CE41" t="str"/>
-      <x:c r="CF41" t="str">
-        <x:v>i18n</x:v>
-      </x:c>
-      <x:c r="CG41" t="str">
-        <x:v>space.onboarding.notice</x:v>
-      </x:c>
-      <x:c r="CH41" t="str">
-        <x:v>SPACE Gallery ver 0.1 / Selected areas are open now. More rooms are under construction.</x:v>
-      </x:c>
-      <x:c r="CI41" t="str">
-        <x:v>SPACE Gallery ver 0.1 / 目前仅开放部分区域，其余展区正在建设中</x:v>
-      </x:c>
+      <x:c r="A41"/>
+      <x:c r="B41"/>
+      <x:c r="C41"/>
+      <x:c r="D41"/>
+      <x:c r="E41"/>
+      <x:c r="F41"/>
+      <x:c r="G41"/>
+      <x:c r="H41"/>
+      <x:c r="I41"/>
+      <x:c r="J41"/>
+      <x:c r="K41"/>
+      <x:c r="L41"/>
+      <x:c r="M41"/>
+      <x:c r="N41"/>
+      <x:c r="O41"/>
+      <x:c r="P41"/>
+      <x:c r="Q41"/>
+      <x:c r="R41"/>
+      <x:c r="S41"/>
+      <x:c r="T41"/>
+      <x:c r="U41"/>
+      <x:c r="V41"/>
+      <x:c r="W41"/>
+      <x:c r="X41"/>
+      <x:c r="Y41"/>
+      <x:c r="Z41"/>
+      <x:c r="AA41"/>
+      <x:c r="AB41"/>
+      <x:c r="AC41"/>
+      <x:c r="AD41"/>
+      <x:c r="AE41"/>
+      <x:c r="AF41"/>
+      <x:c r="AG41"/>
+      <x:c r="AH41"/>
+      <x:c r="AI41"/>
+      <x:c r="AJ41"/>
+      <x:c r="AK41"/>
+      <x:c r="AL41"/>
+      <x:c r="AM41"/>
+      <x:c r="AN41"/>
+      <x:c r="AO41"/>
+      <x:c r="AP41"/>
+      <x:c r="AQ41"/>
+      <x:c r="AR41"/>
+      <x:c r="AS41"/>
+      <x:c r="AT41"/>
+      <x:c r="AU41"/>
+      <x:c r="AV41"/>
+      <x:c r="AW41"/>
+      <x:c r="AX41"/>
+      <x:c r="AY41"/>
+      <x:c r="AZ41"/>
+      <x:c r="BA41"/>
+      <x:c r="BB41"/>
+      <x:c r="BC41"/>
+      <x:c r="BD41"/>
+      <x:c r="BE41"/>
+      <x:c r="BF41"/>
+      <x:c r="BG41"/>
+      <x:c r="BH41"/>
+      <x:c r="BI41"/>
+      <x:c r="BJ41"/>
+      <x:c r="BK41"/>
+      <x:c r="BL41"/>
+      <x:c r="BM41"/>
+      <x:c r="BN41"/>
+      <x:c r="BO41"/>
+      <x:c r="BP41"/>
+      <x:c r="BQ41"/>
+      <x:c r="BR41"/>
+      <x:c r="BS41"/>
+      <x:c r="BT41"/>
+      <x:c r="BU41"/>
+      <x:c r="BV41"/>
+      <x:c r="BW41"/>
+      <x:c r="BX41"/>
+      <x:c r="BY41"/>
+      <x:c r="BZ41"/>
+      <x:c r="CA41"/>
+      <x:c r="CB41"/>
+      <x:c r="CC41"/>
+      <x:c r="CD41"/>
+      <x:c r="CE41"/>
+      <x:c r="CF41"/>
+      <x:c r="CG41"/>
+      <x:c r="CH41"/>
+      <x:c r="CI41"/>
       <x:c r="CJ41" t="str"/>
       <x:c r="CK41" t="str"/>
       <x:c r="CL41" t="str"/>
@@ -11529,10 +11465,10 @@
         <x:v>space.onboarding.look</x:v>
       </x:c>
       <x:c r="CH43" t="str">
-        <x:v>Move the mouse to look; aim at me</x:v>
+        <x:v>Move the mouse to look</x:v>
       </x:c>
       <x:c r="CI43" t="str">
-        <x:v>移动鼠标环顾，对准我</x:v>
+        <x:v>移动鼠标控制视角</x:v>
       </x:c>
       <x:c r="CJ43" t="str"/>
       <x:c r="CK43" t="str"/>
@@ -11545,109 +11481,93 @@
       <x:c r="CR43" t="str"/>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" t="str">
-        <x:v>ui_copy</x:v>
-      </x:c>
-      <x:c r="B44" t="str">
-        <x:v>i18n_space_onboarding_demo</x:v>
-      </x:c>
-      <x:c r="C44" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="D44" t="str">
-        <x:v>3023</x:v>
-      </x:c>
-      <x:c r="E44" t="str"/>
-      <x:c r="F44" t="str"/>
-      <x:c r="G44" t="str"/>
-      <x:c r="H44" t="str"/>
-      <x:c r="I44" t="str"/>
-      <x:c r="J44" t="str"/>
-      <x:c r="K44" t="str"/>
-      <x:c r="L44" t="str"/>
-      <x:c r="M44" t="str"/>
-      <x:c r="N44" t="str"/>
-      <x:c r="O44" t="str"/>
-      <x:c r="P44" t="str"/>
-      <x:c r="Q44" t="str"/>
-      <x:c r="R44" t="str"/>
-      <x:c r="S44" t="str"/>
-      <x:c r="T44" t="str"/>
-      <x:c r="U44" t="str"/>
-      <x:c r="V44" t="str"/>
-      <x:c r="W44" t="str"/>
-      <x:c r="X44" t="str"/>
-      <x:c r="Y44" t="str"/>
-      <x:c r="Z44" t="str"/>
-      <x:c r="AA44" t="str"/>
-      <x:c r="AB44" t="str"/>
-      <x:c r="AC44" t="str"/>
-      <x:c r="AD44" t="str"/>
-      <x:c r="AE44" t="str"/>
-      <x:c r="AF44" t="str"/>
-      <x:c r="AG44" t="str"/>
-      <x:c r="AH44" t="str"/>
-      <x:c r="AI44" t="str"/>
-      <x:c r="AJ44" t="str"/>
-      <x:c r="AK44" t="str"/>
-      <x:c r="AL44" t="str"/>
-      <x:c r="AM44" t="str"/>
-      <x:c r="AN44" t="str"/>
-      <x:c r="AO44" t="str"/>
-      <x:c r="AP44" t="str"/>
-      <x:c r="AQ44" t="str"/>
-      <x:c r="AR44" t="str"/>
-      <x:c r="AS44" t="str"/>
-      <x:c r="AT44" t="str"/>
-      <x:c r="AU44" t="str"/>
-      <x:c r="AV44" t="str"/>
-      <x:c r="AW44" t="str"/>
-      <x:c r="AX44" t="str"/>
-      <x:c r="AY44" t="str"/>
-      <x:c r="AZ44" t="str"/>
-      <x:c r="BA44" t="str"/>
-      <x:c r="BB44" t="str"/>
-      <x:c r="BC44" t="str"/>
-      <x:c r="BD44" t="str"/>
-      <x:c r="BE44" t="str"/>
-      <x:c r="BF44" t="str"/>
-      <x:c r="BG44" t="str"/>
-      <x:c r="BH44" t="str"/>
-      <x:c r="BI44" t="str"/>
-      <x:c r="BJ44" t="str"/>
-      <x:c r="BK44" t="str"/>
-      <x:c r="BL44" t="str"/>
-      <x:c r="BM44" t="str"/>
-      <x:c r="BN44" t="str"/>
-      <x:c r="BO44" t="str"/>
-      <x:c r="BP44" t="str"/>
-      <x:c r="BQ44" t="str"/>
-      <x:c r="BR44" t="str"/>
-      <x:c r="BS44" t="str"/>
-      <x:c r="BT44" t="str"/>
-      <x:c r="BU44" t="str"/>
-      <x:c r="BV44" t="str"/>
-      <x:c r="BW44" t="str"/>
-      <x:c r="BX44" t="str"/>
-      <x:c r="BY44" t="str"/>
-      <x:c r="BZ44" t="str"/>
-      <x:c r="CA44" t="str"/>
-      <x:c r="CB44" t="str"/>
-      <x:c r="CC44" t="str"/>
-      <x:c r="CD44" t="str"/>
-      <x:c r="CE44" t="str"/>
-      <x:c r="CF44" t="str">
-        <x:v>i18n</x:v>
-      </x:c>
-      <x:c r="CG44" t="str">
-        <x:v>space.onboarding.demo</x:v>
-      </x:c>
-      <x:c r="CH44" t="str">
-        <x:v>Aim at this line, then click</x:v>
-      </x:c>
-      <x:c r="CI44" t="str">
-        <x:v>把准星对准我，然后点击</x:v>
-      </x:c>
+      <x:c r="A44"/>
+      <x:c r="B44"/>
+      <x:c r="C44"/>
+      <x:c r="D44"/>
+      <x:c r="E44"/>
+      <x:c r="F44"/>
+      <x:c r="G44"/>
+      <x:c r="H44"/>
+      <x:c r="I44"/>
+      <x:c r="J44"/>
+      <x:c r="K44"/>
+      <x:c r="L44"/>
+      <x:c r="M44"/>
+      <x:c r="N44"/>
+      <x:c r="O44"/>
+      <x:c r="P44"/>
+      <x:c r="Q44"/>
+      <x:c r="R44"/>
+      <x:c r="S44"/>
+      <x:c r="T44"/>
+      <x:c r="U44"/>
+      <x:c r="V44"/>
+      <x:c r="W44"/>
+      <x:c r="X44"/>
+      <x:c r="Y44"/>
+      <x:c r="Z44"/>
+      <x:c r="AA44"/>
+      <x:c r="AB44"/>
+      <x:c r="AC44"/>
+      <x:c r="AD44"/>
+      <x:c r="AE44"/>
+      <x:c r="AF44"/>
+      <x:c r="AG44"/>
+      <x:c r="AH44"/>
+      <x:c r="AI44"/>
+      <x:c r="AJ44"/>
+      <x:c r="AK44"/>
+      <x:c r="AL44"/>
+      <x:c r="AM44"/>
+      <x:c r="AN44"/>
+      <x:c r="AO44"/>
+      <x:c r="AP44"/>
+      <x:c r="AQ44"/>
+      <x:c r="AR44"/>
+      <x:c r="AS44"/>
+      <x:c r="AT44"/>
+      <x:c r="AU44"/>
+      <x:c r="AV44"/>
+      <x:c r="AW44"/>
+      <x:c r="AX44"/>
+      <x:c r="AY44"/>
+      <x:c r="AZ44"/>
+      <x:c r="BA44"/>
+      <x:c r="BB44"/>
+      <x:c r="BC44"/>
+      <x:c r="BD44"/>
+      <x:c r="BE44"/>
+      <x:c r="BF44"/>
+      <x:c r="BG44"/>
+      <x:c r="BH44"/>
+      <x:c r="BI44"/>
+      <x:c r="BJ44"/>
+      <x:c r="BK44"/>
+      <x:c r="BL44"/>
+      <x:c r="BM44"/>
+      <x:c r="BN44"/>
+      <x:c r="BO44"/>
+      <x:c r="BP44"/>
+      <x:c r="BQ44"/>
+      <x:c r="BR44"/>
+      <x:c r="BS44"/>
+      <x:c r="BT44"/>
+      <x:c r="BU44"/>
+      <x:c r="BV44"/>
+      <x:c r="BW44"/>
+      <x:c r="BX44"/>
+      <x:c r="BY44"/>
+      <x:c r="BZ44"/>
+      <x:c r="CA44"/>
+      <x:c r="CB44"/>
+      <x:c r="CC44"/>
+      <x:c r="CD44"/>
+      <x:c r="CE44"/>
+      <x:c r="CF44"/>
+      <x:c r="CG44"/>
+      <x:c r="CH44"/>
+      <x:c r="CI44"/>
       <x:c r="CJ44" t="str"/>
       <x:c r="CK44" t="str"/>
       <x:c r="CL44" t="str"/>
@@ -11659,109 +11579,93 @@
       <x:c r="CR44" t="str"/>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" t="str">
-        <x:v>ui_copy</x:v>
-      </x:c>
-      <x:c r="B45" t="str">
-        <x:v>i18n_space_onboarding_focusTitle</x:v>
-      </x:c>
-      <x:c r="C45" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="D45" t="str">
-        <x:v>3024</x:v>
-      </x:c>
-      <x:c r="E45" t="str"/>
-      <x:c r="F45" t="str"/>
-      <x:c r="G45" t="str"/>
-      <x:c r="H45" t="str"/>
-      <x:c r="I45" t="str"/>
-      <x:c r="J45" t="str"/>
-      <x:c r="K45" t="str"/>
-      <x:c r="L45" t="str"/>
-      <x:c r="M45" t="str"/>
-      <x:c r="N45" t="str"/>
-      <x:c r="O45" t="str"/>
-      <x:c r="P45" t="str"/>
-      <x:c r="Q45" t="str"/>
-      <x:c r="R45" t="str"/>
-      <x:c r="S45" t="str"/>
-      <x:c r="T45" t="str"/>
-      <x:c r="U45" t="str"/>
-      <x:c r="V45" t="str"/>
-      <x:c r="W45" t="str"/>
-      <x:c r="X45" t="str"/>
-      <x:c r="Y45" t="str"/>
-      <x:c r="Z45" t="str"/>
-      <x:c r="AA45" t="str"/>
-      <x:c r="AB45" t="str"/>
-      <x:c r="AC45" t="str"/>
-      <x:c r="AD45" t="str"/>
-      <x:c r="AE45" t="str"/>
-      <x:c r="AF45" t="str"/>
-      <x:c r="AG45" t="str"/>
-      <x:c r="AH45" t="str"/>
-      <x:c r="AI45" t="str"/>
-      <x:c r="AJ45" t="str"/>
-      <x:c r="AK45" t="str"/>
-      <x:c r="AL45" t="str"/>
-      <x:c r="AM45" t="str"/>
-      <x:c r="AN45" t="str"/>
-      <x:c r="AO45" t="str"/>
-      <x:c r="AP45" t="str"/>
-      <x:c r="AQ45" t="str"/>
-      <x:c r="AR45" t="str"/>
-      <x:c r="AS45" t="str"/>
-      <x:c r="AT45" t="str"/>
-      <x:c r="AU45" t="str"/>
-      <x:c r="AV45" t="str"/>
-      <x:c r="AW45" t="str"/>
-      <x:c r="AX45" t="str"/>
-      <x:c r="AY45" t="str"/>
-      <x:c r="AZ45" t="str"/>
-      <x:c r="BA45" t="str"/>
-      <x:c r="BB45" t="str"/>
-      <x:c r="BC45" t="str"/>
-      <x:c r="BD45" t="str"/>
-      <x:c r="BE45" t="str"/>
-      <x:c r="BF45" t="str"/>
-      <x:c r="BG45" t="str"/>
-      <x:c r="BH45" t="str"/>
-      <x:c r="BI45" t="str"/>
-      <x:c r="BJ45" t="str"/>
-      <x:c r="BK45" t="str"/>
-      <x:c r="BL45" t="str"/>
-      <x:c r="BM45" t="str"/>
-      <x:c r="BN45" t="str"/>
-      <x:c r="BO45" t="str"/>
-      <x:c r="BP45" t="str"/>
-      <x:c r="BQ45" t="str"/>
-      <x:c r="BR45" t="str"/>
-      <x:c r="BS45" t="str"/>
-      <x:c r="BT45" t="str"/>
-      <x:c r="BU45" t="str"/>
-      <x:c r="BV45" t="str"/>
-      <x:c r="BW45" t="str"/>
-      <x:c r="BX45" t="str"/>
-      <x:c r="BY45" t="str"/>
-      <x:c r="BZ45" t="str"/>
-      <x:c r="CA45" t="str"/>
-      <x:c r="CB45" t="str"/>
-      <x:c r="CC45" t="str"/>
-      <x:c r="CD45" t="str"/>
-      <x:c r="CE45" t="str"/>
-      <x:c r="CF45" t="str">
-        <x:v>i18n</x:v>
-      </x:c>
-      <x:c r="CG45" t="str">
-        <x:v>space.onboarding.focusTitle</x:v>
-      </x:c>
-      <x:c r="CH45" t="str">
-        <x:v>Exhibits open here</x:v>
-      </x:c>
-      <x:c r="CI45" t="str">
-        <x:v>展品会在这里展开</x:v>
-      </x:c>
+      <x:c r="A45"/>
+      <x:c r="B45"/>
+      <x:c r="C45"/>
+      <x:c r="D45"/>
+      <x:c r="E45"/>
+      <x:c r="F45"/>
+      <x:c r="G45"/>
+      <x:c r="H45"/>
+      <x:c r="I45"/>
+      <x:c r="J45"/>
+      <x:c r="K45"/>
+      <x:c r="L45"/>
+      <x:c r="M45"/>
+      <x:c r="N45"/>
+      <x:c r="O45"/>
+      <x:c r="P45"/>
+      <x:c r="Q45"/>
+      <x:c r="R45"/>
+      <x:c r="S45"/>
+      <x:c r="T45"/>
+      <x:c r="U45"/>
+      <x:c r="V45"/>
+      <x:c r="W45"/>
+      <x:c r="X45"/>
+      <x:c r="Y45"/>
+      <x:c r="Z45"/>
+      <x:c r="AA45"/>
+      <x:c r="AB45"/>
+      <x:c r="AC45"/>
+      <x:c r="AD45"/>
+      <x:c r="AE45"/>
+      <x:c r="AF45"/>
+      <x:c r="AG45"/>
+      <x:c r="AH45"/>
+      <x:c r="AI45"/>
+      <x:c r="AJ45"/>
+      <x:c r="AK45"/>
+      <x:c r="AL45"/>
+      <x:c r="AM45"/>
+      <x:c r="AN45"/>
+      <x:c r="AO45"/>
+      <x:c r="AP45"/>
+      <x:c r="AQ45"/>
+      <x:c r="AR45"/>
+      <x:c r="AS45"/>
+      <x:c r="AT45"/>
+      <x:c r="AU45"/>
+      <x:c r="AV45"/>
+      <x:c r="AW45"/>
+      <x:c r="AX45"/>
+      <x:c r="AY45"/>
+      <x:c r="AZ45"/>
+      <x:c r="BA45"/>
+      <x:c r="BB45"/>
+      <x:c r="BC45"/>
+      <x:c r="BD45"/>
+      <x:c r="BE45"/>
+      <x:c r="BF45"/>
+      <x:c r="BG45"/>
+      <x:c r="BH45"/>
+      <x:c r="BI45"/>
+      <x:c r="BJ45"/>
+      <x:c r="BK45"/>
+      <x:c r="BL45"/>
+      <x:c r="BM45"/>
+      <x:c r="BN45"/>
+      <x:c r="BO45"/>
+      <x:c r="BP45"/>
+      <x:c r="BQ45"/>
+      <x:c r="BR45"/>
+      <x:c r="BS45"/>
+      <x:c r="BT45"/>
+      <x:c r="BU45"/>
+      <x:c r="BV45"/>
+      <x:c r="BW45"/>
+      <x:c r="BX45"/>
+      <x:c r="BY45"/>
+      <x:c r="BZ45"/>
+      <x:c r="CA45"/>
+      <x:c r="CB45"/>
+      <x:c r="CC45"/>
+      <x:c r="CD45"/>
+      <x:c r="CE45"/>
+      <x:c r="CF45"/>
+      <x:c r="CG45"/>
+      <x:c r="CH45"/>
+      <x:c r="CI45"/>
       <x:c r="CJ45" t="str"/>
       <x:c r="CK45" t="str"/>
       <x:c r="CL45" t="str"/>
@@ -11773,109 +11677,93 @@
       <x:c r="CR45" t="str"/>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" t="str">
-        <x:v>ui_copy</x:v>
-      </x:c>
-      <x:c r="B46" t="str">
-        <x:v>i18n_space_onboarding_focusBody</x:v>
-      </x:c>
-      <x:c r="C46" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="D46" t="str">
-        <x:v>3025</x:v>
-      </x:c>
-      <x:c r="E46" t="str"/>
-      <x:c r="F46" t="str"/>
-      <x:c r="G46" t="str"/>
-      <x:c r="H46" t="str"/>
-      <x:c r="I46" t="str"/>
-      <x:c r="J46" t="str"/>
-      <x:c r="K46" t="str"/>
-      <x:c r="L46" t="str"/>
-      <x:c r="M46" t="str"/>
-      <x:c r="N46" t="str"/>
-      <x:c r="O46" t="str"/>
-      <x:c r="P46" t="str"/>
-      <x:c r="Q46" t="str"/>
-      <x:c r="R46" t="str"/>
-      <x:c r="S46" t="str"/>
-      <x:c r="T46" t="str"/>
-      <x:c r="U46" t="str"/>
-      <x:c r="V46" t="str"/>
-      <x:c r="W46" t="str"/>
-      <x:c r="X46" t="str"/>
-      <x:c r="Y46" t="str"/>
-      <x:c r="Z46" t="str"/>
-      <x:c r="AA46" t="str"/>
-      <x:c r="AB46" t="str"/>
-      <x:c r="AC46" t="str"/>
-      <x:c r="AD46" t="str"/>
-      <x:c r="AE46" t="str"/>
-      <x:c r="AF46" t="str"/>
-      <x:c r="AG46" t="str"/>
-      <x:c r="AH46" t="str"/>
-      <x:c r="AI46" t="str"/>
-      <x:c r="AJ46" t="str"/>
-      <x:c r="AK46" t="str"/>
-      <x:c r="AL46" t="str"/>
-      <x:c r="AM46" t="str"/>
-      <x:c r="AN46" t="str"/>
-      <x:c r="AO46" t="str"/>
-      <x:c r="AP46" t="str"/>
-      <x:c r="AQ46" t="str"/>
-      <x:c r="AR46" t="str"/>
-      <x:c r="AS46" t="str"/>
-      <x:c r="AT46" t="str"/>
-      <x:c r="AU46" t="str"/>
-      <x:c r="AV46" t="str"/>
-      <x:c r="AW46" t="str"/>
-      <x:c r="AX46" t="str"/>
-      <x:c r="AY46" t="str"/>
-      <x:c r="AZ46" t="str"/>
-      <x:c r="BA46" t="str"/>
-      <x:c r="BB46" t="str"/>
-      <x:c r="BC46" t="str"/>
-      <x:c r="BD46" t="str"/>
-      <x:c r="BE46" t="str"/>
-      <x:c r="BF46" t="str"/>
-      <x:c r="BG46" t="str"/>
-      <x:c r="BH46" t="str"/>
-      <x:c r="BI46" t="str"/>
-      <x:c r="BJ46" t="str"/>
-      <x:c r="BK46" t="str"/>
-      <x:c r="BL46" t="str"/>
-      <x:c r="BM46" t="str"/>
-      <x:c r="BN46" t="str"/>
-      <x:c r="BO46" t="str"/>
-      <x:c r="BP46" t="str"/>
-      <x:c r="BQ46" t="str"/>
-      <x:c r="BR46" t="str"/>
-      <x:c r="BS46" t="str"/>
-      <x:c r="BT46" t="str"/>
-      <x:c r="BU46" t="str"/>
-      <x:c r="BV46" t="str"/>
-      <x:c r="BW46" t="str"/>
-      <x:c r="BX46" t="str"/>
-      <x:c r="BY46" t="str"/>
-      <x:c r="BZ46" t="str"/>
-      <x:c r="CA46" t="str"/>
-      <x:c r="CB46" t="str"/>
-      <x:c r="CC46" t="str"/>
-      <x:c r="CD46" t="str"/>
-      <x:c r="CE46" t="str"/>
-      <x:c r="CF46" t="str">
-        <x:v>i18n</x:v>
-      </x:c>
-      <x:c r="CG46" t="str">
-        <x:v>space.onboarding.focusBody</x:v>
-      </x:c>
-      <x:c r="CH46" t="str">
-        <x:v>You will learn the story behind each work.</x:v>
-      </x:c>
-      <x:c r="CI46" t="str">
-        <x:v>你将能够了解作品背后的故事</x:v>
-      </x:c>
+      <x:c r="A46"/>
+      <x:c r="B46"/>
+      <x:c r="C46"/>
+      <x:c r="D46"/>
+      <x:c r="E46"/>
+      <x:c r="F46"/>
+      <x:c r="G46"/>
+      <x:c r="H46"/>
+      <x:c r="I46"/>
+      <x:c r="J46"/>
+      <x:c r="K46"/>
+      <x:c r="L46"/>
+      <x:c r="M46"/>
+      <x:c r="N46"/>
+      <x:c r="O46"/>
+      <x:c r="P46"/>
+      <x:c r="Q46"/>
+      <x:c r="R46"/>
+      <x:c r="S46"/>
+      <x:c r="T46"/>
+      <x:c r="U46"/>
+      <x:c r="V46"/>
+      <x:c r="W46"/>
+      <x:c r="X46"/>
+      <x:c r="Y46"/>
+      <x:c r="Z46"/>
+      <x:c r="AA46"/>
+      <x:c r="AB46"/>
+      <x:c r="AC46"/>
+      <x:c r="AD46"/>
+      <x:c r="AE46"/>
+      <x:c r="AF46"/>
+      <x:c r="AG46"/>
+      <x:c r="AH46"/>
+      <x:c r="AI46"/>
+      <x:c r="AJ46"/>
+      <x:c r="AK46"/>
+      <x:c r="AL46"/>
+      <x:c r="AM46"/>
+      <x:c r="AN46"/>
+      <x:c r="AO46"/>
+      <x:c r="AP46"/>
+      <x:c r="AQ46"/>
+      <x:c r="AR46"/>
+      <x:c r="AS46"/>
+      <x:c r="AT46"/>
+      <x:c r="AU46"/>
+      <x:c r="AV46"/>
+      <x:c r="AW46"/>
+      <x:c r="AX46"/>
+      <x:c r="AY46"/>
+      <x:c r="AZ46"/>
+      <x:c r="BA46"/>
+      <x:c r="BB46"/>
+      <x:c r="BC46"/>
+      <x:c r="BD46"/>
+      <x:c r="BE46"/>
+      <x:c r="BF46"/>
+      <x:c r="BG46"/>
+      <x:c r="BH46"/>
+      <x:c r="BI46"/>
+      <x:c r="BJ46"/>
+      <x:c r="BK46"/>
+      <x:c r="BL46"/>
+      <x:c r="BM46"/>
+      <x:c r="BN46"/>
+      <x:c r="BO46"/>
+      <x:c r="BP46"/>
+      <x:c r="BQ46"/>
+      <x:c r="BR46"/>
+      <x:c r="BS46"/>
+      <x:c r="BT46"/>
+      <x:c r="BU46"/>
+      <x:c r="BV46"/>
+      <x:c r="BW46"/>
+      <x:c r="BX46"/>
+      <x:c r="BY46"/>
+      <x:c r="BZ46"/>
+      <x:c r="CA46"/>
+      <x:c r="CB46"/>
+      <x:c r="CC46"/>
+      <x:c r="CD46"/>
+      <x:c r="CE46"/>
+      <x:c r="CF46"/>
+      <x:c r="CG46"/>
+      <x:c r="CH46"/>
+      <x:c r="CI46"/>
       <x:c r="CJ46" t="str"/>
       <x:c r="CK46" t="str"/>
       <x:c r="CL46" t="str"/>
@@ -11887,109 +11775,93 @@
       <x:c r="CR46" t="str"/>
     </x:row>
     <x:row r="47">
-      <x:c r="A47" t="str">
-        <x:v>ui_copy</x:v>
-      </x:c>
-      <x:c r="B47" t="str">
-        <x:v>i18n_space_onboarding_focusExit</x:v>
-      </x:c>
-      <x:c r="C47" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="D47" t="str">
-        <x:v>3026</x:v>
-      </x:c>
-      <x:c r="E47" t="str"/>
-      <x:c r="F47" t="str"/>
-      <x:c r="G47" t="str"/>
-      <x:c r="H47" t="str"/>
-      <x:c r="I47" t="str"/>
-      <x:c r="J47" t="str"/>
-      <x:c r="K47" t="str"/>
-      <x:c r="L47" t="str"/>
-      <x:c r="M47" t="str"/>
-      <x:c r="N47" t="str"/>
-      <x:c r="O47" t="str"/>
-      <x:c r="P47" t="str"/>
-      <x:c r="Q47" t="str"/>
-      <x:c r="R47" t="str"/>
-      <x:c r="S47" t="str"/>
-      <x:c r="T47" t="str"/>
-      <x:c r="U47" t="str"/>
-      <x:c r="V47" t="str"/>
-      <x:c r="W47" t="str"/>
-      <x:c r="X47" t="str"/>
-      <x:c r="Y47" t="str"/>
-      <x:c r="Z47" t="str"/>
-      <x:c r="AA47" t="str"/>
-      <x:c r="AB47" t="str"/>
-      <x:c r="AC47" t="str"/>
-      <x:c r="AD47" t="str"/>
-      <x:c r="AE47" t="str"/>
-      <x:c r="AF47" t="str"/>
-      <x:c r="AG47" t="str"/>
-      <x:c r="AH47" t="str"/>
-      <x:c r="AI47" t="str"/>
-      <x:c r="AJ47" t="str"/>
-      <x:c r="AK47" t="str"/>
-      <x:c r="AL47" t="str"/>
-      <x:c r="AM47" t="str"/>
-      <x:c r="AN47" t="str"/>
-      <x:c r="AO47" t="str"/>
-      <x:c r="AP47" t="str"/>
-      <x:c r="AQ47" t="str"/>
-      <x:c r="AR47" t="str"/>
-      <x:c r="AS47" t="str"/>
-      <x:c r="AT47" t="str"/>
-      <x:c r="AU47" t="str"/>
-      <x:c r="AV47" t="str"/>
-      <x:c r="AW47" t="str"/>
-      <x:c r="AX47" t="str"/>
-      <x:c r="AY47" t="str"/>
-      <x:c r="AZ47" t="str"/>
-      <x:c r="BA47" t="str"/>
-      <x:c r="BB47" t="str"/>
-      <x:c r="BC47" t="str"/>
-      <x:c r="BD47" t="str"/>
-      <x:c r="BE47" t="str"/>
-      <x:c r="BF47" t="str"/>
-      <x:c r="BG47" t="str"/>
-      <x:c r="BH47" t="str"/>
-      <x:c r="BI47" t="str"/>
-      <x:c r="BJ47" t="str"/>
-      <x:c r="BK47" t="str"/>
-      <x:c r="BL47" t="str"/>
-      <x:c r="BM47" t="str"/>
-      <x:c r="BN47" t="str"/>
-      <x:c r="BO47" t="str"/>
-      <x:c r="BP47" t="str"/>
-      <x:c r="BQ47" t="str"/>
-      <x:c r="BR47" t="str"/>
-      <x:c r="BS47" t="str"/>
-      <x:c r="BT47" t="str"/>
-      <x:c r="BU47" t="str"/>
-      <x:c r="BV47" t="str"/>
-      <x:c r="BW47" t="str"/>
-      <x:c r="BX47" t="str"/>
-      <x:c r="BY47" t="str"/>
-      <x:c r="BZ47" t="str"/>
-      <x:c r="CA47" t="str"/>
-      <x:c r="CB47" t="str"/>
-      <x:c r="CC47" t="str"/>
-      <x:c r="CD47" t="str"/>
-      <x:c r="CE47" t="str"/>
-      <x:c r="CF47" t="str">
-        <x:v>i18n</x:v>
-      </x:c>
-      <x:c r="CG47" t="str">
-        <x:v>space.onboarding.focusExit</x:v>
-      </x:c>
-      <x:c r="CH47" t="str">
-        <x:v>Double-click blank space, or click the top space button to return to SPACE</x:v>
-      </x:c>
-      <x:c r="CI47" t="str">
-        <x:v>双击空白，或点击顶部 space 回到 SPACE</x:v>
-      </x:c>
+      <x:c r="A47"/>
+      <x:c r="B47"/>
+      <x:c r="C47"/>
+      <x:c r="D47"/>
+      <x:c r="E47"/>
+      <x:c r="F47"/>
+      <x:c r="G47"/>
+      <x:c r="H47"/>
+      <x:c r="I47"/>
+      <x:c r="J47"/>
+      <x:c r="K47"/>
+      <x:c r="L47"/>
+      <x:c r="M47"/>
+      <x:c r="N47"/>
+      <x:c r="O47"/>
+      <x:c r="P47"/>
+      <x:c r="Q47"/>
+      <x:c r="R47"/>
+      <x:c r="S47"/>
+      <x:c r="T47"/>
+      <x:c r="U47"/>
+      <x:c r="V47"/>
+      <x:c r="W47"/>
+      <x:c r="X47"/>
+      <x:c r="Y47"/>
+      <x:c r="Z47"/>
+      <x:c r="AA47"/>
+      <x:c r="AB47"/>
+      <x:c r="AC47"/>
+      <x:c r="AD47"/>
+      <x:c r="AE47"/>
+      <x:c r="AF47"/>
+      <x:c r="AG47"/>
+      <x:c r="AH47"/>
+      <x:c r="AI47"/>
+      <x:c r="AJ47"/>
+      <x:c r="AK47"/>
+      <x:c r="AL47"/>
+      <x:c r="AM47"/>
+      <x:c r="AN47"/>
+      <x:c r="AO47"/>
+      <x:c r="AP47"/>
+      <x:c r="AQ47"/>
+      <x:c r="AR47"/>
+      <x:c r="AS47"/>
+      <x:c r="AT47"/>
+      <x:c r="AU47"/>
+      <x:c r="AV47"/>
+      <x:c r="AW47"/>
+      <x:c r="AX47"/>
+      <x:c r="AY47"/>
+      <x:c r="AZ47"/>
+      <x:c r="BA47"/>
+      <x:c r="BB47"/>
+      <x:c r="BC47"/>
+      <x:c r="BD47"/>
+      <x:c r="BE47"/>
+      <x:c r="BF47"/>
+      <x:c r="BG47"/>
+      <x:c r="BH47"/>
+      <x:c r="BI47"/>
+      <x:c r="BJ47"/>
+      <x:c r="BK47"/>
+      <x:c r="BL47"/>
+      <x:c r="BM47"/>
+      <x:c r="BN47"/>
+      <x:c r="BO47"/>
+      <x:c r="BP47"/>
+      <x:c r="BQ47"/>
+      <x:c r="BR47"/>
+      <x:c r="BS47"/>
+      <x:c r="BT47"/>
+      <x:c r="BU47"/>
+      <x:c r="BV47"/>
+      <x:c r="BW47"/>
+      <x:c r="BX47"/>
+      <x:c r="BY47"/>
+      <x:c r="BZ47"/>
+      <x:c r="CA47"/>
+      <x:c r="CB47"/>
+      <x:c r="CC47"/>
+      <x:c r="CD47"/>
+      <x:c r="CE47"/>
+      <x:c r="CF47"/>
+      <x:c r="CG47"/>
+      <x:c r="CH47"/>
+      <x:c r="CI47"/>
       <x:c r="CJ47" t="str"/>
       <x:c r="CK47" t="str"/>
       <x:c r="CL47" t="str"/>
@@ -12001,109 +11873,93 @@
       <x:c r="CR47" t="str"/>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" t="str">
-        <x:v>ui_copy</x:v>
-      </x:c>
-      <x:c r="B48" t="str">
-        <x:v>i18n_space_onboarding_esc</x:v>
-      </x:c>
-      <x:c r="C48" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="D48" t="str">
-        <x:v>3027</x:v>
-      </x:c>
-      <x:c r="E48" t="str"/>
-      <x:c r="F48" t="str"/>
-      <x:c r="G48" t="str"/>
-      <x:c r="H48" t="str"/>
-      <x:c r="I48" t="str"/>
-      <x:c r="J48" t="str"/>
-      <x:c r="K48" t="str"/>
-      <x:c r="L48" t="str"/>
-      <x:c r="M48" t="str"/>
-      <x:c r="N48" t="str"/>
-      <x:c r="O48" t="str"/>
-      <x:c r="P48" t="str"/>
-      <x:c r="Q48" t="str"/>
-      <x:c r="R48" t="str"/>
-      <x:c r="S48" t="str"/>
-      <x:c r="T48" t="str"/>
-      <x:c r="U48" t="str"/>
-      <x:c r="V48" t="str"/>
-      <x:c r="W48" t="str"/>
-      <x:c r="X48" t="str"/>
-      <x:c r="Y48" t="str"/>
-      <x:c r="Z48" t="str"/>
-      <x:c r="AA48" t="str"/>
-      <x:c r="AB48" t="str"/>
-      <x:c r="AC48" t="str"/>
-      <x:c r="AD48" t="str"/>
-      <x:c r="AE48" t="str"/>
-      <x:c r="AF48" t="str"/>
-      <x:c r="AG48" t="str"/>
-      <x:c r="AH48" t="str"/>
-      <x:c r="AI48" t="str"/>
-      <x:c r="AJ48" t="str"/>
-      <x:c r="AK48" t="str"/>
-      <x:c r="AL48" t="str"/>
-      <x:c r="AM48" t="str"/>
-      <x:c r="AN48" t="str"/>
-      <x:c r="AO48" t="str"/>
-      <x:c r="AP48" t="str"/>
-      <x:c r="AQ48" t="str"/>
-      <x:c r="AR48" t="str"/>
-      <x:c r="AS48" t="str"/>
-      <x:c r="AT48" t="str"/>
-      <x:c r="AU48" t="str"/>
-      <x:c r="AV48" t="str"/>
-      <x:c r="AW48" t="str"/>
-      <x:c r="AX48" t="str"/>
-      <x:c r="AY48" t="str"/>
-      <x:c r="AZ48" t="str"/>
-      <x:c r="BA48" t="str"/>
-      <x:c r="BB48" t="str"/>
-      <x:c r="BC48" t="str"/>
-      <x:c r="BD48" t="str"/>
-      <x:c r="BE48" t="str"/>
-      <x:c r="BF48" t="str"/>
-      <x:c r="BG48" t="str"/>
-      <x:c r="BH48" t="str"/>
-      <x:c r="BI48" t="str"/>
-      <x:c r="BJ48" t="str"/>
-      <x:c r="BK48" t="str"/>
-      <x:c r="BL48" t="str"/>
-      <x:c r="BM48" t="str"/>
-      <x:c r="BN48" t="str"/>
-      <x:c r="BO48" t="str"/>
-      <x:c r="BP48" t="str"/>
-      <x:c r="BQ48" t="str"/>
-      <x:c r="BR48" t="str"/>
-      <x:c r="BS48" t="str"/>
-      <x:c r="BT48" t="str"/>
-      <x:c r="BU48" t="str"/>
-      <x:c r="BV48" t="str"/>
-      <x:c r="BW48" t="str"/>
-      <x:c r="BX48" t="str"/>
-      <x:c r="BY48" t="str"/>
-      <x:c r="BZ48" t="str"/>
-      <x:c r="CA48" t="str"/>
-      <x:c r="CB48" t="str"/>
-      <x:c r="CC48" t="str"/>
-      <x:c r="CD48" t="str"/>
-      <x:c r="CE48" t="str"/>
-      <x:c r="CF48" t="str">
-        <x:v>i18n</x:v>
-      </x:c>
-      <x:c r="CG48" t="str">
-        <x:v>space.onboarding.esc</x:v>
-      </x:c>
-      <x:c r="CH48" t="str">
-        <x:v>Press Esc to release the mouse</x:v>
-      </x:c>
-      <x:c r="CI48" t="str">
-        <x:v>按 Esc 呼出鼠标</x:v>
-      </x:c>
+      <x:c r="A48"/>
+      <x:c r="B48"/>
+      <x:c r="C48"/>
+      <x:c r="D48"/>
+      <x:c r="E48"/>
+      <x:c r="F48"/>
+      <x:c r="G48"/>
+      <x:c r="H48"/>
+      <x:c r="I48"/>
+      <x:c r="J48"/>
+      <x:c r="K48"/>
+      <x:c r="L48"/>
+      <x:c r="M48"/>
+      <x:c r="N48"/>
+      <x:c r="O48"/>
+      <x:c r="P48"/>
+      <x:c r="Q48"/>
+      <x:c r="R48"/>
+      <x:c r="S48"/>
+      <x:c r="T48"/>
+      <x:c r="U48"/>
+      <x:c r="V48"/>
+      <x:c r="W48"/>
+      <x:c r="X48"/>
+      <x:c r="Y48"/>
+      <x:c r="Z48"/>
+      <x:c r="AA48"/>
+      <x:c r="AB48"/>
+      <x:c r="AC48"/>
+      <x:c r="AD48"/>
+      <x:c r="AE48"/>
+      <x:c r="AF48"/>
+      <x:c r="AG48"/>
+      <x:c r="AH48"/>
+      <x:c r="AI48"/>
+      <x:c r="AJ48"/>
+      <x:c r="AK48"/>
+      <x:c r="AL48"/>
+      <x:c r="AM48"/>
+      <x:c r="AN48"/>
+      <x:c r="AO48"/>
+      <x:c r="AP48"/>
+      <x:c r="AQ48"/>
+      <x:c r="AR48"/>
+      <x:c r="AS48"/>
+      <x:c r="AT48"/>
+      <x:c r="AU48"/>
+      <x:c r="AV48"/>
+      <x:c r="AW48"/>
+      <x:c r="AX48"/>
+      <x:c r="AY48"/>
+      <x:c r="AZ48"/>
+      <x:c r="BA48"/>
+      <x:c r="BB48"/>
+      <x:c r="BC48"/>
+      <x:c r="BD48"/>
+      <x:c r="BE48"/>
+      <x:c r="BF48"/>
+      <x:c r="BG48"/>
+      <x:c r="BH48"/>
+      <x:c r="BI48"/>
+      <x:c r="BJ48"/>
+      <x:c r="BK48"/>
+      <x:c r="BL48"/>
+      <x:c r="BM48"/>
+      <x:c r="BN48"/>
+      <x:c r="BO48"/>
+      <x:c r="BP48"/>
+      <x:c r="BQ48"/>
+      <x:c r="BR48"/>
+      <x:c r="BS48"/>
+      <x:c r="BT48"/>
+      <x:c r="BU48"/>
+      <x:c r="BV48"/>
+      <x:c r="BW48"/>
+      <x:c r="BX48"/>
+      <x:c r="BY48"/>
+      <x:c r="BZ48"/>
+      <x:c r="CA48"/>
+      <x:c r="CB48"/>
+      <x:c r="CC48"/>
+      <x:c r="CD48"/>
+      <x:c r="CE48"/>
+      <x:c r="CF48"/>
+      <x:c r="CG48"/>
+      <x:c r="CH48"/>
+      <x:c r="CI48"/>
       <x:c r="CJ48" t="str"/>
       <x:c r="CK48" t="str"/>
       <x:c r="CL48" t="str"/>
@@ -12115,109 +11971,93 @@
       <x:c r="CR48" t="str"/>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" t="str">
-        <x:v>ui_copy</x:v>
-      </x:c>
-      <x:c r="B49" t="str">
-        <x:v>i18n_space_onboarding_relock</x:v>
-      </x:c>
-      <x:c r="C49" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="D49" t="str">
-        <x:v>3028</x:v>
-      </x:c>
-      <x:c r="E49" t="str"/>
-      <x:c r="F49" t="str"/>
-      <x:c r="G49" t="str"/>
-      <x:c r="H49" t="str"/>
-      <x:c r="I49" t="str"/>
-      <x:c r="J49" t="str"/>
-      <x:c r="K49" t="str"/>
-      <x:c r="L49" t="str"/>
-      <x:c r="M49" t="str"/>
-      <x:c r="N49" t="str"/>
-      <x:c r="O49" t="str"/>
-      <x:c r="P49" t="str"/>
-      <x:c r="Q49" t="str"/>
-      <x:c r="R49" t="str"/>
-      <x:c r="S49" t="str"/>
-      <x:c r="T49" t="str"/>
-      <x:c r="U49" t="str"/>
-      <x:c r="V49" t="str"/>
-      <x:c r="W49" t="str"/>
-      <x:c r="X49" t="str"/>
-      <x:c r="Y49" t="str"/>
-      <x:c r="Z49" t="str"/>
-      <x:c r="AA49" t="str"/>
-      <x:c r="AB49" t="str"/>
-      <x:c r="AC49" t="str"/>
-      <x:c r="AD49" t="str"/>
-      <x:c r="AE49" t="str"/>
-      <x:c r="AF49" t="str"/>
-      <x:c r="AG49" t="str"/>
-      <x:c r="AH49" t="str"/>
-      <x:c r="AI49" t="str"/>
-      <x:c r="AJ49" t="str"/>
-      <x:c r="AK49" t="str"/>
-      <x:c r="AL49" t="str"/>
-      <x:c r="AM49" t="str"/>
-      <x:c r="AN49" t="str"/>
-      <x:c r="AO49" t="str"/>
-      <x:c r="AP49" t="str"/>
-      <x:c r="AQ49" t="str"/>
-      <x:c r="AR49" t="str"/>
-      <x:c r="AS49" t="str"/>
-      <x:c r="AT49" t="str"/>
-      <x:c r="AU49" t="str"/>
-      <x:c r="AV49" t="str"/>
-      <x:c r="AW49" t="str"/>
-      <x:c r="AX49" t="str"/>
-      <x:c r="AY49" t="str"/>
-      <x:c r="AZ49" t="str"/>
-      <x:c r="BA49" t="str"/>
-      <x:c r="BB49" t="str"/>
-      <x:c r="BC49" t="str"/>
-      <x:c r="BD49" t="str"/>
-      <x:c r="BE49" t="str"/>
-      <x:c r="BF49" t="str"/>
-      <x:c r="BG49" t="str"/>
-      <x:c r="BH49" t="str"/>
-      <x:c r="BI49" t="str"/>
-      <x:c r="BJ49" t="str"/>
-      <x:c r="BK49" t="str"/>
-      <x:c r="BL49" t="str"/>
-      <x:c r="BM49" t="str"/>
-      <x:c r="BN49" t="str"/>
-      <x:c r="BO49" t="str"/>
-      <x:c r="BP49" t="str"/>
-      <x:c r="BQ49" t="str"/>
-      <x:c r="BR49" t="str"/>
-      <x:c r="BS49" t="str"/>
-      <x:c r="BT49" t="str"/>
-      <x:c r="BU49" t="str"/>
-      <x:c r="BV49" t="str"/>
-      <x:c r="BW49" t="str"/>
-      <x:c r="BX49" t="str"/>
-      <x:c r="BY49" t="str"/>
-      <x:c r="BZ49" t="str"/>
-      <x:c r="CA49" t="str"/>
-      <x:c r="CB49" t="str"/>
-      <x:c r="CC49" t="str"/>
-      <x:c r="CD49" t="str"/>
-      <x:c r="CE49" t="str"/>
-      <x:c r="CF49" t="str">
-        <x:v>i18n</x:v>
-      </x:c>
-      <x:c r="CG49" t="str">
-        <x:v>space.onboarding.relock</x:v>
-      </x:c>
-      <x:c r="CH49" t="str">
-        <x:v>Click an empty area to control the view again</x:v>
-      </x:c>
-      <x:c r="CI49" t="str">
-        <x:v>点击空白区域重新控制视角</x:v>
-      </x:c>
+      <x:c r="A49"/>
+      <x:c r="B49"/>
+      <x:c r="C49"/>
+      <x:c r="D49"/>
+      <x:c r="E49"/>
+      <x:c r="F49"/>
+      <x:c r="G49"/>
+      <x:c r="H49"/>
+      <x:c r="I49"/>
+      <x:c r="J49"/>
+      <x:c r="K49"/>
+      <x:c r="L49"/>
+      <x:c r="M49"/>
+      <x:c r="N49"/>
+      <x:c r="O49"/>
+      <x:c r="P49"/>
+      <x:c r="Q49"/>
+      <x:c r="R49"/>
+      <x:c r="S49"/>
+      <x:c r="T49"/>
+      <x:c r="U49"/>
+      <x:c r="V49"/>
+      <x:c r="W49"/>
+      <x:c r="X49"/>
+      <x:c r="Y49"/>
+      <x:c r="Z49"/>
+      <x:c r="AA49"/>
+      <x:c r="AB49"/>
+      <x:c r="AC49"/>
+      <x:c r="AD49"/>
+      <x:c r="AE49"/>
+      <x:c r="AF49"/>
+      <x:c r="AG49"/>
+      <x:c r="AH49"/>
+      <x:c r="AI49"/>
+      <x:c r="AJ49"/>
+      <x:c r="AK49"/>
+      <x:c r="AL49"/>
+      <x:c r="AM49"/>
+      <x:c r="AN49"/>
+      <x:c r="AO49"/>
+      <x:c r="AP49"/>
+      <x:c r="AQ49"/>
+      <x:c r="AR49"/>
+      <x:c r="AS49"/>
+      <x:c r="AT49"/>
+      <x:c r="AU49"/>
+      <x:c r="AV49"/>
+      <x:c r="AW49"/>
+      <x:c r="AX49"/>
+      <x:c r="AY49"/>
+      <x:c r="AZ49"/>
+      <x:c r="BA49"/>
+      <x:c r="BB49"/>
+      <x:c r="BC49"/>
+      <x:c r="BD49"/>
+      <x:c r="BE49"/>
+      <x:c r="BF49"/>
+      <x:c r="BG49"/>
+      <x:c r="BH49"/>
+      <x:c r="BI49"/>
+      <x:c r="BJ49"/>
+      <x:c r="BK49"/>
+      <x:c r="BL49"/>
+      <x:c r="BM49"/>
+      <x:c r="BN49"/>
+      <x:c r="BO49"/>
+      <x:c r="BP49"/>
+      <x:c r="BQ49"/>
+      <x:c r="BR49"/>
+      <x:c r="BS49"/>
+      <x:c r="BT49"/>
+      <x:c r="BU49"/>
+      <x:c r="BV49"/>
+      <x:c r="BW49"/>
+      <x:c r="BX49"/>
+      <x:c r="BY49"/>
+      <x:c r="BZ49"/>
+      <x:c r="CA49"/>
+      <x:c r="CB49"/>
+      <x:c r="CC49"/>
+      <x:c r="CD49"/>
+      <x:c r="CE49"/>
+      <x:c r="CF49"/>
+      <x:c r="CG49"/>
+      <x:c r="CH49"/>
+      <x:c r="CI49"/>
       <x:c r="CJ49" t="str"/>
       <x:c r="CK49" t="str"/>
       <x:c r="CL49" t="str"/>
@@ -12229,109 +12069,93 @@
       <x:c r="CR49" t="str"/>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" t="str">
-        <x:v>ui_copy</x:v>
-      </x:c>
-      <x:c r="B50" t="str">
-        <x:v>i18n_space_onboarding_done</x:v>
-      </x:c>
-      <x:c r="C50" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="D50" t="str">
-        <x:v>3029</x:v>
-      </x:c>
-      <x:c r="E50" t="str"/>
-      <x:c r="F50" t="str"/>
-      <x:c r="G50" t="str"/>
-      <x:c r="H50" t="str"/>
-      <x:c r="I50" t="str"/>
-      <x:c r="J50" t="str"/>
-      <x:c r="K50" t="str"/>
-      <x:c r="L50" t="str"/>
-      <x:c r="M50" t="str"/>
-      <x:c r="N50" t="str"/>
-      <x:c r="O50" t="str"/>
-      <x:c r="P50" t="str"/>
-      <x:c r="Q50" t="str"/>
-      <x:c r="R50" t="str"/>
-      <x:c r="S50" t="str"/>
-      <x:c r="T50" t="str"/>
-      <x:c r="U50" t="str"/>
-      <x:c r="V50" t="str"/>
-      <x:c r="W50" t="str"/>
-      <x:c r="X50" t="str"/>
-      <x:c r="Y50" t="str"/>
-      <x:c r="Z50" t="str"/>
-      <x:c r="AA50" t="str"/>
-      <x:c r="AB50" t="str"/>
-      <x:c r="AC50" t="str"/>
-      <x:c r="AD50" t="str"/>
-      <x:c r="AE50" t="str"/>
-      <x:c r="AF50" t="str"/>
-      <x:c r="AG50" t="str"/>
-      <x:c r="AH50" t="str"/>
-      <x:c r="AI50" t="str"/>
-      <x:c r="AJ50" t="str"/>
-      <x:c r="AK50" t="str"/>
-      <x:c r="AL50" t="str"/>
-      <x:c r="AM50" t="str"/>
-      <x:c r="AN50" t="str"/>
-      <x:c r="AO50" t="str"/>
-      <x:c r="AP50" t="str"/>
-      <x:c r="AQ50" t="str"/>
-      <x:c r="AR50" t="str"/>
-      <x:c r="AS50" t="str"/>
-      <x:c r="AT50" t="str"/>
-      <x:c r="AU50" t="str"/>
-      <x:c r="AV50" t="str"/>
-      <x:c r="AW50" t="str"/>
-      <x:c r="AX50" t="str"/>
-      <x:c r="AY50" t="str"/>
-      <x:c r="AZ50" t="str"/>
-      <x:c r="BA50" t="str"/>
-      <x:c r="BB50" t="str"/>
-      <x:c r="BC50" t="str"/>
-      <x:c r="BD50" t="str"/>
-      <x:c r="BE50" t="str"/>
-      <x:c r="BF50" t="str"/>
-      <x:c r="BG50" t="str"/>
-      <x:c r="BH50" t="str"/>
-      <x:c r="BI50" t="str"/>
-      <x:c r="BJ50" t="str"/>
-      <x:c r="BK50" t="str"/>
-      <x:c r="BL50" t="str"/>
-      <x:c r="BM50" t="str"/>
-      <x:c r="BN50" t="str"/>
-      <x:c r="BO50" t="str"/>
-      <x:c r="BP50" t="str"/>
-      <x:c r="BQ50" t="str"/>
-      <x:c r="BR50" t="str"/>
-      <x:c r="BS50" t="str"/>
-      <x:c r="BT50" t="str"/>
-      <x:c r="BU50" t="str"/>
-      <x:c r="BV50" t="str"/>
-      <x:c r="BW50" t="str"/>
-      <x:c r="BX50" t="str"/>
-      <x:c r="BY50" t="str"/>
-      <x:c r="BZ50" t="str"/>
-      <x:c r="CA50" t="str"/>
-      <x:c r="CB50" t="str"/>
-      <x:c r="CC50" t="str"/>
-      <x:c r="CD50" t="str"/>
-      <x:c r="CE50" t="str"/>
-      <x:c r="CF50" t="str">
-        <x:v>i18n</x:v>
-      </x:c>
-      <x:c r="CG50" t="str">
-        <x:v>space.onboarding.done</x:v>
-      </x:c>
-      <x:c r="CH50" t="str">
-        <x:v>Follow the path to SPACE</x:v>
-      </x:c>
-      <x:c r="CI50" t="str">
-        <x:v>顺着道路前往 SPACE 吧</x:v>
-      </x:c>
+      <x:c r="A50"/>
+      <x:c r="B50"/>
+      <x:c r="C50"/>
+      <x:c r="D50"/>
+      <x:c r="E50"/>
+      <x:c r="F50"/>
+      <x:c r="G50"/>
+      <x:c r="H50"/>
+      <x:c r="I50"/>
+      <x:c r="J50"/>
+      <x:c r="K50"/>
+      <x:c r="L50"/>
+      <x:c r="M50"/>
+      <x:c r="N50"/>
+      <x:c r="O50"/>
+      <x:c r="P50"/>
+      <x:c r="Q50"/>
+      <x:c r="R50"/>
+      <x:c r="S50"/>
+      <x:c r="T50"/>
+      <x:c r="U50"/>
+      <x:c r="V50"/>
+      <x:c r="W50"/>
+      <x:c r="X50"/>
+      <x:c r="Y50"/>
+      <x:c r="Z50"/>
+      <x:c r="AA50"/>
+      <x:c r="AB50"/>
+      <x:c r="AC50"/>
+      <x:c r="AD50"/>
+      <x:c r="AE50"/>
+      <x:c r="AF50"/>
+      <x:c r="AG50"/>
+      <x:c r="AH50"/>
+      <x:c r="AI50"/>
+      <x:c r="AJ50"/>
+      <x:c r="AK50"/>
+      <x:c r="AL50"/>
+      <x:c r="AM50"/>
+      <x:c r="AN50"/>
+      <x:c r="AO50"/>
+      <x:c r="AP50"/>
+      <x:c r="AQ50"/>
+      <x:c r="AR50"/>
+      <x:c r="AS50"/>
+      <x:c r="AT50"/>
+      <x:c r="AU50"/>
+      <x:c r="AV50"/>
+      <x:c r="AW50"/>
+      <x:c r="AX50"/>
+      <x:c r="AY50"/>
+      <x:c r="AZ50"/>
+      <x:c r="BA50"/>
+      <x:c r="BB50"/>
+      <x:c r="BC50"/>
+      <x:c r="BD50"/>
+      <x:c r="BE50"/>
+      <x:c r="BF50"/>
+      <x:c r="BG50"/>
+      <x:c r="BH50"/>
+      <x:c r="BI50"/>
+      <x:c r="BJ50"/>
+      <x:c r="BK50"/>
+      <x:c r="BL50"/>
+      <x:c r="BM50"/>
+      <x:c r="BN50"/>
+      <x:c r="BO50"/>
+      <x:c r="BP50"/>
+      <x:c r="BQ50"/>
+      <x:c r="BR50"/>
+      <x:c r="BS50"/>
+      <x:c r="BT50"/>
+      <x:c r="BU50"/>
+      <x:c r="BV50"/>
+      <x:c r="BW50"/>
+      <x:c r="BX50"/>
+      <x:c r="BY50"/>
+      <x:c r="BZ50"/>
+      <x:c r="CA50"/>
+      <x:c r="CB50"/>
+      <x:c r="CC50"/>
+      <x:c r="CD50"/>
+      <x:c r="CE50"/>
+      <x:c r="CF50"/>
+      <x:c r="CG50"/>
+      <x:c r="CH50"/>
+      <x:c r="CI50"/>
       <x:c r="CJ50" t="str"/>
       <x:c r="CK50" t="str"/>
       <x:c r="CL50" t="str"/>

</xml_diff>

<commit_message>
content: ground profile and academic studies in reviewed PDF sources
</commit_message>
<xml_diff>
--- a/docs/assets/space-exhibit-index.xlsx
+++ b/docs/assets/space-exhibit-index.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="education" sheetId="1" r:id="R068516fa9ac04fad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="professional_practice" sheetId="2" r:id="R2207edc4af454bbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="personal_archive" sheetId="3" r:id="R0c4b1f37ad7044e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="explore" sheetId="4" r:id="R22d8fc92f72a4073"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="education" sheetId="1" r:id="R3820d79a09664a7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="professional_practice" sheetId="2" r:id="Red77ef147d444084"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="personal_archive" sheetId="3" r:id="R41dc363b687f4aa5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="explore" sheetId="4" r:id="R74e5ea22ea3e4a31"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -645,19 +645,23 @@
         <x:v>建筑图纸、数字模型、图像序列</x:v>
       </x:c>
       <x:c r="X2" t="str">
-        <x:v>Concept, design, model, presentation</x:v>
+        <x:v>Individual academic project · Pratt ARCH 402</x:v>
       </x:c>
       <x:c r="Y2" t="str">
-        <x:v>概念、设计、建模、表达</x:v>
+        <x:v>个人学术作品 · Pratt ARCH 402</x:v>
       </x:c>
       <x:c r="Z2" t="str">
-        <x:v>Student portfolio exhibit</x:v>
+        <x:v>Academic proposal · Skyhive 2021 shortlist</x:v>
       </x:c>
       <x:c r="AA2" t="str">
-        <x:v>学生作品集展品</x:v>
-      </x:c>
-      <x:c r="AB2" t="str"/>
-      <x:c r="AC2" t="str"/>
+        <x:v>学术方案 · 入围 Skyhive 2021</x:v>
+      </x:c>
+      <x:c r="AB2" t="str">
+        <x:v>Instructors: Kathleen Dunne, Michael Trencher</x:v>
+      </x:c>
+      <x:c r="AC2" t="str">
+        <x:v>指导教师：Kathleen Dunne、Michael Trencher</x:v>
+      </x:c>
       <x:c r="AD2" t="str"/>
       <x:c r="AE2" t="str"/>
       <x:c r="AF2" t="str">
@@ -700,22 +704,22 @@
         <x:v>Tree Habitat 在这里作为学生阶段建筑作品呈现，而不是已建成或商业项目。重点是学习阶段的设计命题：如何把生态结构转译成剖面、动线、功能叠合和建筑表达。</x:v>
       </x:c>
       <x:c r="AS2" t="str">
-        <x:v>The project should read as academic architecture and spatial design research, with the model and images serving the concept rather than claiming finished delivery.</x:v>
+        <x:v>Concept, design, model, presentation</x:v>
       </x:c>
       <x:c r="AT2" t="str">
-        <x:v>这个项目应被读作 academic architecture 和 spatial design research；模型与图片服务于概念，而不是包装成成熟交付项目。</x:v>
+        <x:v>概念、设计、建模、表达</x:v>
       </x:c>
       <x:c r="AU2" t="str">
-        <x:v>Education layer / Student Room entry for architecture studio work, image boards, model views, and concept notes.</x:v>
+        <x:v>student work/mixed use highrise</x:v>
       </x:c>
       <x:c r="AV2" t="str">
-        <x:v>Education layer / Student Room 条目，用于承载建筑 studio 作品、图像板、模型视角和概念说明。</x:v>
+        <x:v>学生作品 / 复合功能高层</x:v>
       </x:c>
       <x:c r="AW2" t="str">
-        <x:v>Mobile keeps this entry text-and-image first. The 3D model remains a desktop Focus artifact and is not shown in the phone view.</x:v>
+        <x:v>Student portfolio exhibit</x:v>
       </x:c>
       <x:c r="AX2" t="str">
-        <x:v>移动端保持文字和图片优先。3D 模型保留给桌面端 Focus，不在手机页面展示。</x:v>
+        <x:v>学生作品集展品</x:v>
       </x:c>
       <x:c r="AY2" t="str">
         <x:v>/exhibits/arch_treehabitat/focus_arch_treehabitat.glb</x:v>
@@ -861,7 +865,7 @@
       </x:c>
       <x:c r="Q3" t="str"/>
       <x:c r="R3" t="str">
-        <x:v>2025</x:v>
+        <x:v>2025–2026</x:v>
       </x:c>
       <x:c r="S3" t="str"/>
       <x:c r="T3" t="str">
@@ -902,13 +906,13 @@
         <x:v>围绕深圳日常空间系统的城市研究与展览模型研究</x:v>
       </x:c>
       <x:c r="AI3" t="str">
-        <x:v>Study</x:v>
+        <x:v>Architecture</x:v>
       </x:c>
       <x:c r="AJ3" t="str">
-        <x:v>stage-student</x:v>
+        <x:v>stage-work</x:v>
       </x:c>
       <x:c r="AK3" t="str">
-        <x:v>Education</x:v>
+        <x:v>Professional Practice</x:v>
       </x:c>
       <x:c r="AL3" t="str">
         <x:v>model</x:v>
@@ -932,22 +936,22 @@
         <x:v>UABB Exhibit 位于城市研究与展览设计之间。它研究日常街道片段、商业节奏、门槛空间和服务空间如何被压缩成一个像空间档案一样可阅读的模型。</x:v>
       </x:c>
       <x:c r="AS3" t="str">
-        <x:v>The work should read as research translated into space: observation, mapping, model logic, and exhibition language working together.</x:v>
+        <x:v>Research, mapping, modeling, exhibition narrative</x:v>
       </x:c>
       <x:c r="AT3" t="str">
-        <x:v>这个作品应被读作被转译为空间的研究：观察、mapping、模型逻辑和展览语言共同工作。</x:v>
+        <x:v>研究、mapping、建模、展览叙事</x:v>
       </x:c>
       <x:c r="AU3" t="str">
-        <x:v>Education layer / Urban research entry for model-based exhibition thinking and future research boards.</x:v>
+        <x:v>UABB exhibition proposal / urban typology research</x:v>
       </x:c>
       <x:c r="AV3" t="str">
-        <x:v>Education layer / Urban research 条目，用于承载基于模型的展览思考和未来研究板内容。</x:v>
+        <x:v>UABB 展览方案 / 城市类型研究</x:v>
       </x:c>
       <x:c r="AW3" t="str">
-        <x:v>Mobile keeps the project text-first while desktop SPACE carries the heavier model artifact.</x:v>
+        <x:v>Biennale exhibit archive</x:v>
       </x:c>
       <x:c r="AX3" t="str">
-        <x:v>移动端先保持文字优先；较重的模型展品由桌面端 SPACE 承载。</x:v>
+        <x:v>双年展展品档案</x:v>
       </x:c>
       <x:c r="AY3" t="str">
         <x:v>/exhibits/arch_uabb_exhibit/focus_arch_uabb_exhibit.glb</x:v>
@@ -1152,22 +1156,22 @@
         <x:v>过程动画想象一个预先设计好的建筑如何被快速搭建：水泥打印墙体以 0.9 米为阶段逐层生长，预制结构件和组件在关键节点介入，整套系统可以在完整建造前快速迭代。</x:v>
       </x:c>
       <x:c r="AS4" t="str">
-        <x:v>The work should feel compact and process-led: model first, one animation second, with no extra documentation noise.</x:v>
+        <x:v>Design, model, fabrication workflow, video presentation</x:v>
       </x:c>
       <x:c r="AT4" t="str">
-        <x:v>这个作品应该保持紧凑并以过程为主：先看模型，再看一个动画，不加入多余文档噪音。</x:v>
+        <x:v>设计、建模、制造流程、视频表达</x:v>
       </x:c>
       <x:c r="AU4" t="str">
-        <x:v>Education layer / Fabrication entry for physical modeling, 3D printing, and process video.</x:v>
+        <x:v>student work / 3D printing architecture animation</x:v>
       </x:c>
       <x:c r="AV4" t="str">
-        <x:v>Education layer / Fabrication 条目，用于呈现实体模型、3D 打印和过程视频。</x:v>
+        <x:v>学生作品 / 3D 打印建筑动画</x:v>
       </x:c>
       <x:c r="AW4" t="str">
-        <x:v>Mobile describes the artifact; desktop Focus shows the rotatable model and MP4 process animation.</x:v>
+        <x:v>Portfolio exhibit draft</x:v>
       </x:c>
       <x:c r="AX4" t="str">
-        <x:v>移动端描述作品；桌面端 Focus 展示可旋转模型和 MP4 过程动画。</x:v>
+        <x:v>作品集展品草案</x:v>
       </x:c>
       <x:c r="AY4" t="str">
         <x:v>/exhibits/arch_3d_printing_architecture/focus_arch_3d_printing_architecture.glb</x:v>
@@ -1244,7 +1248,7 @@
         <x:v>project-02</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>40</x:v>
@@ -1392,7 +1396,7 @@
         <x:v>project-12</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>140</x:v>
@@ -1549,17 +1553,17 @@
         <x:v>Education</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>Education</x:v>
+        <x:v>教育经历</x:v>
       </x:c>
       <x:c r="G7" t="str"/>
       <x:c r="H7" t="str"/>
       <x:c r="I7" t="str"/>
       <x:c r="J7" t="str"/>
       <x:c r="K7" t="str">
-        <x:v>From Pratt's architecture foundation to Columbia's research-led spatial experiments, school shaped how I read scale, sequence, image, and systems.</x:v>
+        <x:v>Architectural education spanning building design, interior space and research into public life.</x:v>
       </x:c>
       <x:c r="L7" t="str">
-        <x:v>从 Pratt 的建筑基础训练到 Columbia 更研究导向的空间实验，教育经历构成了我理解尺度、叙事、图像和系统的底层方法。</x:v>
+        <x:v>从建筑与室内空间设计，到公共生活与空间叙事研究。</x:v>
       </x:c>
       <x:c r="M7" t="str"/>
       <x:c r="N7" t="str"/>
@@ -1633,36 +1637,42 @@
       <x:c r="BR7" t="str"/>
       <x:c r="BS7" t="str"/>
       <x:c r="BT7" t="str">
-        <x:v>Pratt Institute / Columbia University</x:v>
+        <x:v>Pratt Institute · Columbia University GSAPP</x:v>
       </x:c>
       <x:c r="BU7" t="str">
-        <x:v>Pratt Institute / Columbia University</x:v>
+        <x:v>Pratt Institute · Columbia University GSAPP</x:v>
       </x:c>
       <x:c r="BV7" t="str">
-        <x:v>Built a shared language across drawings, sections, models, material studies, and narrative presentation.
-Connected research studios, spatial prototypes, and AI-assisted design into one working method.
-Focused on how diagrams, model photography, renderings, and walk-throughs can explain a spatial idea together.</x:v>
+        <x:v>2022–2023 · Columbia University GSAPP, Manhattan, New York · M.S. Advanced Architectural Design.
+2017–2022 · Pratt Institute School of Architecture, Brooklyn, New York · Bachelor of Architecture (2022), minor in Interior Design.</x:v>
       </x:c>
       <x:c r="BW7" t="str">
-        <x:v>以建筑 studio 训练建立平面、剖面、模型、材料和叙事表达的共同语言。
-把研究型课程、空间原型和 AI 辅助设计放进同一套创作方法里。
-关注 diagram、模型照片、渲染和 walk-through 之间如何共同讲清一个空间概念。</x:v>
+        <x:v>2022–2023 · Columbia University GSAPP，纽约曼哈顿 · M.S. Advanced Architectural Design（高级建筑设计理学硕士）。
+2017–2022 · Pratt Institute School of Architecture，纽约布鲁克林 · 2022 年获建筑学学士，辅修室内设计。</x:v>
       </x:c>
       <x:c r="BX7" t="str">
-        <x:v>Pratt becomes a foundation archive for studio intensity, drawing logic, and model language.
-Columbia becomes an experiment archive for spatial research, computation, and AI visual methods.
-Each academic node can connect to SPACE through project images, short statements, and walkable exhibits.</x:v>
+        <x:v>2022 · Sovereignty of Voices · Columbia studio with Wentao LIU; work shown in the Parallel UN exhibition, September 1–30, 2022.
+2022 · Liberation of Antarctica · Individual speculative redevelopment study at McMurdo Station.
+2021 · Tree Habitat · Individual mixed-use tower study in Shenzhen; shortlisted in Skyhive 2021.
+2021 · Three Circles In · Guangzhou urban acupuncture degree project with Tiancheng YE.
+2020 · The Home Alive · Individual modular housing study in Levittown; honorable mention in HOME 2020.
+2019 · Sky Village · Multigenerational housing in Brooklyn with Tiancheng YE.
+2019 · Storyline Studio · Individual film-studio design in Manhattan.</x:v>
       </x:c>
       <x:c r="BY7" t="str">
-        <x:v>Pratt 作为基础档案区，呈现训练强度、图面逻辑和模型语言。
-Columbia 作为实验档案区，呈现空间研究、计算设计和 AI 视觉方法。
-每个学术节点会以项目图像、短 statement 和可漫游展品连接到 SPACE。</x:v>
+        <x:v>2022 · Sovereignty of Voices · 与 Wentao LIU 合作的 Columbia studio 作品；于 2022 年 9 月 1–30 日在 Parallel UN 展览中展出。
+2022 · Liberation of Antarctica · 位于麦克默多站的个人推想型更新研究。
+2021 · Tree Habitat · 深圳复合功能塔楼个人研究；入围 Skyhive 2021。
+2021 · Three Circles In · 与 Tiancheng YE 合作的广州城市针灸毕业设计。
+2020 · The Home Alive · Levittown 模块化住宅个人研究；获 HOME 2020 荣誉提名。
+2019 · Sky Village · 与 Tiancheng YE 合作的布鲁克林多代共居设计。
+2019 · Storyline Studio · 曼哈顿电影工作室个人设计。</x:v>
       </x:c>
       <x:c r="BZ7" t="str">
-        <x:v>In SPACE, this can become two archive walls: Pratt as foundational training, Columbia as research and experimentation.</x:v>
+        <x:v>Academic proposals explore spatial relationships through drawings, models and narrative; they are presented as design studies.</x:v>
       </x:c>
       <x:c r="CA7" t="str">
-        <x:v>SPACE 中可以做成两段展墙：Pratt 作为基础训练档案，Columbia 作为研究和实验档案。</x:v>
+        <x:v>这些学术方案通过图纸、模型与叙事研究空间关系，均以设计研究的属性呈现。</x:v>
       </x:c>
       <x:c r="CB7" t="str"/>
       <x:c r="CC7" t="str"/>
@@ -1682,6 +1692,990 @@
       <x:c r="CQ7" t="str"/>
       <x:c r="CR7" t="str"/>
     </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>project</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>sovereignty-of-voices</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>Sovereignty of Voices</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>Sovereignty of Voices</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>Sovereignty of Voices</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>Sovereignty of Voices</x:v>
+      </x:c>
+      <x:c r="I8"/>
+      <x:c r="J8"/>
+      <x:c r="K8" t="str">
+        <x:v>A public landscape and theater proposal for the UN north lawn, connecting underground theaters, an accessible landscape and a roof through a central circulation space.</x:v>
+      </x:c>
+      <x:c r="L8" t="str">
+        <x:v>为联合国北草坪提出的公共景观与剧场方案，以中心交通空间连接地下剧场、可进入的地景与屋顶。</x:v>
+      </x:c>
+      <x:c r="M8"/>
+      <x:c r="N8"/>
+      <x:c r="O8"/>
+      <x:c r="P8"/>
+      <x:c r="Q8" t="str">
+        <x:v>Tianyi WANG; Wentao LIU</x:v>
+      </x:c>
+      <x:c r="R8" t="str">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="S8"/>
+      <x:c r="T8"/>
+      <x:c r="U8"/>
+      <x:c r="V8"/>
+      <x:c r="W8"/>
+      <x:c r="X8"/>
+      <x:c r="Y8"/>
+      <x:c r="Z8"/>
+      <x:c r="AA8"/>
+      <x:c r="AB8"/>
+      <x:c r="AC8"/>
+      <x:c r="AD8"/>
+      <x:c r="AE8"/>
+      <x:c r="AF8" t="str">
+        <x:v>2022 · Manhattan, New York</x:v>
+      </x:c>
+      <x:c r="AG8" t="str">
+        <x:v>2022 · Columbia GSAPP · Summer studio</x:v>
+      </x:c>
+      <x:c r="AH8" t="str">
+        <x:v>2022 · Columbia GSAPP · 夏季 studio</x:v>
+      </x:c>
+      <x:c r="AI8" t="str">
+        <x:v>Study</x:v>
+      </x:c>
+      <x:c r="AJ8" t="str">
+        <x:v>stage-student</x:v>
+      </x:c>
+      <x:c r="AK8" t="str">
+        <x:v>Education</x:v>
+      </x:c>
+      <x:c r="AL8" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="AM8" t="str">
+        <x:v>Text study</x:v>
+      </x:c>
+      <x:c r="AN8" t="str">
+        <x:v>文字研究</x:v>
+      </x:c>
+      <x:c r="AO8" t="str">
+        <x:v>A public landscape and theater proposal for the UN north lawn, connecting underground theaters, an accessible landscape and a roof through a central circulation space.</x:v>
+      </x:c>
+      <x:c r="AP8" t="str">
+        <x:v>为联合国北草坪提出的公共景观与剧场方案，以中心交通空间连接地下剧场、可进入的地景与屋顶。</x:v>
+      </x:c>
+      <x:c r="AQ8" t="str">
+        <x:v>Columbia GSAPP · Summer studio. Site: Manhattan, New York. Credits: Tianyi WANG; Wentao LIU.</x:v>
+      </x:c>
+      <x:c r="AR8" t="str">
+        <x:v>Columbia GSAPP · 夏季 studio。项目地点：纽约曼哈顿。作者：Tianyi WANG; Wentao LIU。</x:v>
+      </x:c>
+      <x:c r="AS8" t="str">
+        <x:v>Columbia GSAPP · Summer studio</x:v>
+      </x:c>
+      <x:c r="AT8" t="str">
+        <x:v>Columbia GSAPP · 夏季 studio</x:v>
+      </x:c>
+      <x:c r="AU8" t="str">
+        <x:v>Site: Manhattan, New York</x:v>
+      </x:c>
+      <x:c r="AV8" t="str">
+        <x:v>项目地点：纽约曼哈顿</x:v>
+      </x:c>
+      <x:c r="AW8" t="str">
+        <x:v>Academic design proposal.</x:v>
+      </x:c>
+      <x:c r="AX8" t="str">
+        <x:v>学术设计方案。</x:v>
+      </x:c>
+      <x:c r="AY8"/>
+      <x:c r="AZ8"/>
+      <x:c r="BA8"/>
+      <x:c r="BB8"/>
+      <x:c r="BC8"/>
+      <x:c r="BD8"/>
+      <x:c r="BE8"/>
+      <x:c r="BF8"/>
+      <x:c r="BG8"/>
+      <x:c r="BH8"/>
+      <x:c r="BI8"/>
+      <x:c r="BJ8"/>
+      <x:c r="BK8"/>
+      <x:c r="BL8"/>
+      <x:c r="BM8"/>
+      <x:c r="BN8"/>
+      <x:c r="BO8"/>
+      <x:c r="BP8"/>
+      <x:c r="BQ8"/>
+      <x:c r="BR8"/>
+      <x:c r="BS8"/>
+      <x:c r="BT8"/>
+      <x:c r="BU8"/>
+      <x:c r="BV8"/>
+      <x:c r="BW8"/>
+      <x:c r="BX8"/>
+      <x:c r="BY8"/>
+      <x:c r="BZ8"/>
+      <x:c r="CA8"/>
+      <x:c r="CB8"/>
+      <x:c r="CC8"/>
+      <x:c r="CD8"/>
+      <x:c r="CE8"/>
+      <x:c r="CF8"/>
+      <x:c r="CG8"/>
+      <x:c r="CH8"/>
+      <x:c r="CI8"/>
+      <x:c r="CJ8"/>
+      <x:c r="CK8"/>
+      <x:c r="CL8"/>
+      <x:c r="CM8" t="str">
+        <x:v>Source: Portfolio - Tianyi WANG - 20 mb.pdf, PDF page 3. Website models and images await author delivery.</x:v>
+      </x:c>
+      <x:c r="CN8"/>
+      <x:c r="CO8"/>
+      <x:c r="CP8"/>
+      <x:c r="CQ8"/>
+      <x:c r="CR8" t="str">
+        <x:v>2026-09-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>project</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>liberation-of-antarctica</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>Liberation of Antarctica</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>Liberation of Antarctica</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>Liberation of Antarctica</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>Liberation of Antarctica</x:v>
+      </x:c>
+      <x:c r="I9"/>
+      <x:c r="J9"/>
+      <x:c r="K9" t="str">
+        <x:v>A speculative phased plan for reducing human occupation in Antarctica, consolidating research stations and eventually shifting toward automated remote observation after 2100.</x:v>
+      </x:c>
+      <x:c r="L9" t="str">
+        <x:v>推想分阶段减少人类对南极的占用，整合科考站，并在 2100 年之后逐渐转向自动化远程观测。</x:v>
+      </x:c>
+      <x:c r="M9"/>
+      <x:c r="N9"/>
+      <x:c r="O9"/>
+      <x:c r="P9"/>
+      <x:c r="Q9" t="str">
+        <x:v>Tianyi WANG</x:v>
+      </x:c>
+      <x:c r="R9" t="str">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="S9"/>
+      <x:c r="T9"/>
+      <x:c r="U9"/>
+      <x:c r="V9"/>
+      <x:c r="W9"/>
+      <x:c r="X9"/>
+      <x:c r="Y9"/>
+      <x:c r="Z9"/>
+      <x:c r="AA9"/>
+      <x:c r="AB9"/>
+      <x:c r="AC9"/>
+      <x:c r="AD9"/>
+      <x:c r="AE9"/>
+      <x:c r="AF9" t="str">
+        <x:v>2022 · McMurdo Station, Antarctica</x:v>
+      </x:c>
+      <x:c r="AG9" t="str">
+        <x:v>2022 · Columbia GSAPP · Fall studio · Individual work</x:v>
+      </x:c>
+      <x:c r="AH9" t="str">
+        <x:v>2022 · Columbia GSAPP · 秋季 studio · 个人作品</x:v>
+      </x:c>
+      <x:c r="AI9" t="str">
+        <x:v>Study</x:v>
+      </x:c>
+      <x:c r="AJ9" t="str">
+        <x:v>stage-student</x:v>
+      </x:c>
+      <x:c r="AK9" t="str">
+        <x:v>Education</x:v>
+      </x:c>
+      <x:c r="AL9" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="AM9" t="str">
+        <x:v>Text study</x:v>
+      </x:c>
+      <x:c r="AN9" t="str">
+        <x:v>文字研究</x:v>
+      </x:c>
+      <x:c r="AO9" t="str">
+        <x:v>A speculative phased plan for reducing human occupation in Antarctica, consolidating research stations and eventually shifting toward automated remote observation after 2100.</x:v>
+      </x:c>
+      <x:c r="AP9" t="str">
+        <x:v>推想分阶段减少人类对南极的占用，整合科考站，并在 2100 年之后逐渐转向自动化远程观测。</x:v>
+      </x:c>
+      <x:c r="AQ9" t="str">
+        <x:v>Columbia GSAPP · Fall studio · Individual work. Site: McMurdo Station, Antarctica. Credits: Tianyi WANG.</x:v>
+      </x:c>
+      <x:c r="AR9" t="str">
+        <x:v>Columbia GSAPP · 秋季 studio · 个人作品。项目地点：南极麦克默多站。作者：Tianyi WANG。</x:v>
+      </x:c>
+      <x:c r="AS9" t="str">
+        <x:v>Columbia GSAPP · Fall studio · Individual work</x:v>
+      </x:c>
+      <x:c r="AT9" t="str">
+        <x:v>Columbia GSAPP · 秋季 studio · 个人作品</x:v>
+      </x:c>
+      <x:c r="AU9" t="str">
+        <x:v>Site: McMurdo Station, Antarctica</x:v>
+      </x:c>
+      <x:c r="AV9" t="str">
+        <x:v>项目地点：南极麦克默多站</x:v>
+      </x:c>
+      <x:c r="AW9" t="str">
+        <x:v>Academic design proposal.</x:v>
+      </x:c>
+      <x:c r="AX9" t="str">
+        <x:v>学术设计方案。</x:v>
+      </x:c>
+      <x:c r="AY9"/>
+      <x:c r="AZ9"/>
+      <x:c r="BA9"/>
+      <x:c r="BB9"/>
+      <x:c r="BC9"/>
+      <x:c r="BD9"/>
+      <x:c r="BE9"/>
+      <x:c r="BF9"/>
+      <x:c r="BG9"/>
+      <x:c r="BH9"/>
+      <x:c r="BI9"/>
+      <x:c r="BJ9"/>
+      <x:c r="BK9"/>
+      <x:c r="BL9"/>
+      <x:c r="BM9"/>
+      <x:c r="BN9"/>
+      <x:c r="BO9"/>
+      <x:c r="BP9"/>
+      <x:c r="BQ9"/>
+      <x:c r="BR9"/>
+      <x:c r="BS9"/>
+      <x:c r="BT9"/>
+      <x:c r="BU9"/>
+      <x:c r="BV9"/>
+      <x:c r="BW9"/>
+      <x:c r="BX9"/>
+      <x:c r="BY9"/>
+      <x:c r="BZ9"/>
+      <x:c r="CA9"/>
+      <x:c r="CB9"/>
+      <x:c r="CC9"/>
+      <x:c r="CD9"/>
+      <x:c r="CE9"/>
+      <x:c r="CF9"/>
+      <x:c r="CG9"/>
+      <x:c r="CH9"/>
+      <x:c r="CI9"/>
+      <x:c r="CJ9"/>
+      <x:c r="CK9"/>
+      <x:c r="CL9"/>
+      <x:c r="CM9" t="str">
+        <x:v>Source: Portfolio - Tianyi WANG - 20 mb.pdf, PDF page 11. Website models and images await author delivery.</x:v>
+      </x:c>
+      <x:c r="CN9"/>
+      <x:c r="CO9"/>
+      <x:c r="CP9"/>
+      <x:c r="CQ9"/>
+      <x:c r="CR9" t="str">
+        <x:v>2026-09-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>project</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>three-circles-in</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>Three Circles In</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>Three Circles In</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>Three Circles In</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>Three Circles In</x:v>
+      </x:c>
+      <x:c r="I10"/>
+      <x:c r="J10"/>
+      <x:c r="K10" t="str">
+        <x:v>An urban acupuncture study reconnecting buildings, infrastructure and overlooked communal spaces through a continuous system of public landforms.</x:v>
+      </x:c>
+      <x:c r="L10" t="str">
+        <x:v>以城市针灸为方法，通过连续的公共地形系统重新连接建筑、基础设施与被忽视的社区公共空间。</x:v>
+      </x:c>
+      <x:c r="M10"/>
+      <x:c r="N10"/>
+      <x:c r="O10"/>
+      <x:c r="P10"/>
+      <x:c r="Q10" t="str">
+        <x:v>Tianyi WANG; Tiancheng YE</x:v>
+      </x:c>
+      <x:c r="R10" t="str">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="S10"/>
+      <x:c r="T10"/>
+      <x:c r="U10"/>
+      <x:c r="V10"/>
+      <x:c r="W10"/>
+      <x:c r="X10"/>
+      <x:c r="Y10"/>
+      <x:c r="Z10"/>
+      <x:c r="AA10"/>
+      <x:c r="AB10"/>
+      <x:c r="AC10"/>
+      <x:c r="AD10"/>
+      <x:c r="AE10"/>
+      <x:c r="AF10" t="str">
+        <x:v>2021 · Guangzhou, China</x:v>
+      </x:c>
+      <x:c r="AG10" t="str">
+        <x:v>2021 · Pratt · Degree project · Group work</x:v>
+      </x:c>
+      <x:c r="AH10" t="str">
+        <x:v>2021 · Pratt · 毕业设计 · 合作作品</x:v>
+      </x:c>
+      <x:c r="AI10" t="str">
+        <x:v>Study</x:v>
+      </x:c>
+      <x:c r="AJ10" t="str">
+        <x:v>stage-student</x:v>
+      </x:c>
+      <x:c r="AK10" t="str">
+        <x:v>Education</x:v>
+      </x:c>
+      <x:c r="AL10" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="AM10" t="str">
+        <x:v>Text study</x:v>
+      </x:c>
+      <x:c r="AN10" t="str">
+        <x:v>文字研究</x:v>
+      </x:c>
+      <x:c r="AO10" t="str">
+        <x:v>An urban acupuncture study reconnecting buildings, infrastructure and overlooked communal spaces through a continuous system of public landforms.</x:v>
+      </x:c>
+      <x:c r="AP10" t="str">
+        <x:v>以城市针灸为方法，通过连续的公共地形系统重新连接建筑、基础设施与被忽视的社区公共空间。</x:v>
+      </x:c>
+      <x:c r="AQ10" t="str">
+        <x:v>Pratt · Degree project · Group work. Site: Guangzhou, China. Credits: Tianyi WANG; Tiancheng YE.</x:v>
+      </x:c>
+      <x:c r="AR10" t="str">
+        <x:v>Pratt · 毕业设计 · 合作作品。项目地点：中国广州。作者：Tianyi WANG; Tiancheng YE。</x:v>
+      </x:c>
+      <x:c r="AS10" t="str">
+        <x:v>Pratt · Degree project · Group work</x:v>
+      </x:c>
+      <x:c r="AT10" t="str">
+        <x:v>Pratt · 毕业设计 · 合作作品</x:v>
+      </x:c>
+      <x:c r="AU10" t="str">
+        <x:v>Site: Guangzhou, China</x:v>
+      </x:c>
+      <x:c r="AV10" t="str">
+        <x:v>项目地点：中国广州</x:v>
+      </x:c>
+      <x:c r="AW10" t="str">
+        <x:v>Academic design proposal.</x:v>
+      </x:c>
+      <x:c r="AX10" t="str">
+        <x:v>学术设计方案。</x:v>
+      </x:c>
+      <x:c r="AY10"/>
+      <x:c r="AZ10"/>
+      <x:c r="BA10"/>
+      <x:c r="BB10"/>
+      <x:c r="BC10"/>
+      <x:c r="BD10"/>
+      <x:c r="BE10"/>
+      <x:c r="BF10"/>
+      <x:c r="BG10"/>
+      <x:c r="BH10"/>
+      <x:c r="BI10"/>
+      <x:c r="BJ10"/>
+      <x:c r="BK10"/>
+      <x:c r="BL10"/>
+      <x:c r="BM10"/>
+      <x:c r="BN10"/>
+      <x:c r="BO10"/>
+      <x:c r="BP10"/>
+      <x:c r="BQ10"/>
+      <x:c r="BR10"/>
+      <x:c r="BS10"/>
+      <x:c r="BT10"/>
+      <x:c r="BU10"/>
+      <x:c r="BV10"/>
+      <x:c r="BW10"/>
+      <x:c r="BX10"/>
+      <x:c r="BY10"/>
+      <x:c r="BZ10"/>
+      <x:c r="CA10"/>
+      <x:c r="CB10"/>
+      <x:c r="CC10"/>
+      <x:c r="CD10"/>
+      <x:c r="CE10"/>
+      <x:c r="CF10"/>
+      <x:c r="CG10"/>
+      <x:c r="CH10"/>
+      <x:c r="CI10"/>
+      <x:c r="CJ10"/>
+      <x:c r="CK10"/>
+      <x:c r="CL10"/>
+      <x:c r="CM10" t="str">
+        <x:v>Source: Portfolio - Tianyi WANG - 20 mb.pdf, PDF page 20. Website models and images await author delivery.</x:v>
+      </x:c>
+      <x:c r="CN10"/>
+      <x:c r="CO10"/>
+      <x:c r="CP10"/>
+      <x:c r="CQ10"/>
+      <x:c r="CR10" t="str">
+        <x:v>2026-09-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>project</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>the-home-alive</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>The Home Alive</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>The Home Alive</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>The Home Alive</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>The Home Alive</x:v>
+      </x:c>
+      <x:c r="I11"/>
+      <x:c r="J11"/>
+      <x:c r="K11" t="str">
+        <x:v>A modular housing proposal with an adaptable structural frame and replaceable floor and facade panels, allowing homes to change with the needs of a family. Honorable mention, HOME 2020.</x:v>
+      </x:c>
+      <x:c r="L11" t="str">
+        <x:v>以可调整的结构框架及可替换的楼面、立面面板组织模块化住宅，使住宅随家庭需求变化。获 HOME 2020 荣誉提名。</x:v>
+      </x:c>
+      <x:c r="M11"/>
+      <x:c r="N11"/>
+      <x:c r="O11"/>
+      <x:c r="P11"/>
+      <x:c r="Q11" t="str">
+        <x:v>Tianyi WANG</x:v>
+      </x:c>
+      <x:c r="R11" t="str">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="S11"/>
+      <x:c r="T11"/>
+      <x:c r="U11"/>
+      <x:c r="V11"/>
+      <x:c r="W11"/>
+      <x:c r="X11"/>
+      <x:c r="Y11"/>
+      <x:c r="Z11"/>
+      <x:c r="AA11"/>
+      <x:c r="AB11"/>
+      <x:c r="AC11"/>
+      <x:c r="AD11"/>
+      <x:c r="AE11"/>
+      <x:c r="AF11" t="str">
+        <x:v>2020 · Levittown</x:v>
+      </x:c>
+      <x:c r="AG11" t="str">
+        <x:v>2020 · Pratt ARCH 401 · Individual work</x:v>
+      </x:c>
+      <x:c r="AH11" t="str">
+        <x:v>2020 · Pratt ARCH 401 · 个人作品</x:v>
+      </x:c>
+      <x:c r="AI11" t="str">
+        <x:v>Study</x:v>
+      </x:c>
+      <x:c r="AJ11" t="str">
+        <x:v>stage-student</x:v>
+      </x:c>
+      <x:c r="AK11" t="str">
+        <x:v>Education</x:v>
+      </x:c>
+      <x:c r="AL11" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="AM11" t="str">
+        <x:v>Text study</x:v>
+      </x:c>
+      <x:c r="AN11" t="str">
+        <x:v>文字研究</x:v>
+      </x:c>
+      <x:c r="AO11" t="str">
+        <x:v>A modular housing proposal with an adaptable structural frame and replaceable floor and facade panels, allowing homes to change with the needs of a family. Honorable mention, HOME 2020.</x:v>
+      </x:c>
+      <x:c r="AP11" t="str">
+        <x:v>以可调整的结构框架及可替换的楼面、立面面板组织模块化住宅，使住宅随家庭需求变化。获 HOME 2020 荣誉提名。</x:v>
+      </x:c>
+      <x:c r="AQ11" t="str">
+        <x:v>Pratt ARCH 401 · Individual work. Site: Levittown. Credits: Tianyi WANG.</x:v>
+      </x:c>
+      <x:c r="AR11" t="str">
+        <x:v>Pratt ARCH 401 · 个人作品。项目地点：Levittown。作者：Tianyi WANG。</x:v>
+      </x:c>
+      <x:c r="AS11" t="str">
+        <x:v>Pratt ARCH 401 · Individual work</x:v>
+      </x:c>
+      <x:c r="AT11" t="str">
+        <x:v>Pratt ARCH 401 · 个人作品</x:v>
+      </x:c>
+      <x:c r="AU11" t="str">
+        <x:v>Site: Levittown</x:v>
+      </x:c>
+      <x:c r="AV11" t="str">
+        <x:v>项目地点：Levittown</x:v>
+      </x:c>
+      <x:c r="AW11" t="str">
+        <x:v>Academic design proposal.</x:v>
+      </x:c>
+      <x:c r="AX11" t="str">
+        <x:v>学术设计方案。</x:v>
+      </x:c>
+      <x:c r="AY11"/>
+      <x:c r="AZ11"/>
+      <x:c r="BA11"/>
+      <x:c r="BB11"/>
+      <x:c r="BC11"/>
+      <x:c r="BD11"/>
+      <x:c r="BE11"/>
+      <x:c r="BF11"/>
+      <x:c r="BG11"/>
+      <x:c r="BH11"/>
+      <x:c r="BI11"/>
+      <x:c r="BJ11"/>
+      <x:c r="BK11"/>
+      <x:c r="BL11"/>
+      <x:c r="BM11"/>
+      <x:c r="BN11"/>
+      <x:c r="BO11"/>
+      <x:c r="BP11"/>
+      <x:c r="BQ11"/>
+      <x:c r="BR11"/>
+      <x:c r="BS11"/>
+      <x:c r="BT11"/>
+      <x:c r="BU11"/>
+      <x:c r="BV11"/>
+      <x:c r="BW11"/>
+      <x:c r="BX11"/>
+      <x:c r="BY11"/>
+      <x:c r="BZ11"/>
+      <x:c r="CA11"/>
+      <x:c r="CB11"/>
+      <x:c r="CC11"/>
+      <x:c r="CD11"/>
+      <x:c r="CE11"/>
+      <x:c r="CF11"/>
+      <x:c r="CG11"/>
+      <x:c r="CH11"/>
+      <x:c r="CI11"/>
+      <x:c r="CJ11"/>
+      <x:c r="CK11"/>
+      <x:c r="CL11"/>
+      <x:c r="CM11" t="str">
+        <x:v>Source: Portfolio - Tianyi WANG - 20 mb.pdf, PDF page 28. Website models and images await author delivery.</x:v>
+      </x:c>
+      <x:c r="CN11"/>
+      <x:c r="CO11"/>
+      <x:c r="CP11"/>
+      <x:c r="CQ11"/>
+      <x:c r="CR11" t="str">
+        <x:v>2026-09-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>project</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>sky-village</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>Sky Village</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>Sky Village</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>Sky Village</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>Sky Village</x:v>
+      </x:c>
+      <x:c r="I12"/>
+      <x:c r="J12"/>
+      <x:c r="K12" t="str">
+        <x:v>A multigenerational co-housing proposal distributing shared facilities and circulation across a residential complex while retaining private space within each home.</x:v>
+      </x:c>
+      <x:c r="L12" t="str">
+        <x:v>多代共居住宅方案，将共享设施和交通路径分布在住区中，同时保留各住宅单元的私密空间。</x:v>
+      </x:c>
+      <x:c r="M12"/>
+      <x:c r="N12"/>
+      <x:c r="O12"/>
+      <x:c r="P12"/>
+      <x:c r="Q12" t="str">
+        <x:v>Tianyi WANG; Tiancheng YE</x:v>
+      </x:c>
+      <x:c r="R12" t="str">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="S12"/>
+      <x:c r="T12"/>
+      <x:c r="U12"/>
+      <x:c r="V12"/>
+      <x:c r="W12"/>
+      <x:c r="X12"/>
+      <x:c r="Y12"/>
+      <x:c r="Z12"/>
+      <x:c r="AA12"/>
+      <x:c r="AB12"/>
+      <x:c r="AC12"/>
+      <x:c r="AD12"/>
+      <x:c r="AE12"/>
+      <x:c r="AF12" t="str">
+        <x:v>2019 · Brooklyn, New York</x:v>
+      </x:c>
+      <x:c r="AG12" t="str">
+        <x:v>2019 · Pratt ARCH 301 · Group work</x:v>
+      </x:c>
+      <x:c r="AH12" t="str">
+        <x:v>2019 · Pratt ARCH 301 · 合作作品</x:v>
+      </x:c>
+      <x:c r="AI12" t="str">
+        <x:v>Study</x:v>
+      </x:c>
+      <x:c r="AJ12" t="str">
+        <x:v>stage-student</x:v>
+      </x:c>
+      <x:c r="AK12" t="str">
+        <x:v>Education</x:v>
+      </x:c>
+      <x:c r="AL12" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="AM12" t="str">
+        <x:v>Text study</x:v>
+      </x:c>
+      <x:c r="AN12" t="str">
+        <x:v>文字研究</x:v>
+      </x:c>
+      <x:c r="AO12" t="str">
+        <x:v>A multigenerational co-housing proposal distributing shared facilities and circulation across a residential complex while retaining private space within each home.</x:v>
+      </x:c>
+      <x:c r="AP12" t="str">
+        <x:v>多代共居住宅方案，将共享设施和交通路径分布在住区中，同时保留各住宅单元的私密空间。</x:v>
+      </x:c>
+      <x:c r="AQ12" t="str">
+        <x:v>Pratt ARCH 301 · Group work. Site: Brooklyn, New York. Credits: Tianyi WANG; Tiancheng YE.</x:v>
+      </x:c>
+      <x:c r="AR12" t="str">
+        <x:v>Pratt ARCH 301 · 合作作品。项目地点：纽约布鲁克林。作者：Tianyi WANG; Tiancheng YE。</x:v>
+      </x:c>
+      <x:c r="AS12" t="str">
+        <x:v>Pratt ARCH 301 · Group work</x:v>
+      </x:c>
+      <x:c r="AT12" t="str">
+        <x:v>Pratt ARCH 301 · 合作作品</x:v>
+      </x:c>
+      <x:c r="AU12" t="str">
+        <x:v>Site: Brooklyn, New York</x:v>
+      </x:c>
+      <x:c r="AV12" t="str">
+        <x:v>项目地点：纽约布鲁克林</x:v>
+      </x:c>
+      <x:c r="AW12" t="str">
+        <x:v>Academic design proposal.</x:v>
+      </x:c>
+      <x:c r="AX12" t="str">
+        <x:v>学术设计方案。</x:v>
+      </x:c>
+      <x:c r="AY12"/>
+      <x:c r="AZ12"/>
+      <x:c r="BA12"/>
+      <x:c r="BB12"/>
+      <x:c r="BC12"/>
+      <x:c r="BD12"/>
+      <x:c r="BE12"/>
+      <x:c r="BF12"/>
+      <x:c r="BG12"/>
+      <x:c r="BH12"/>
+      <x:c r="BI12"/>
+      <x:c r="BJ12"/>
+      <x:c r="BK12"/>
+      <x:c r="BL12"/>
+      <x:c r="BM12"/>
+      <x:c r="BN12"/>
+      <x:c r="BO12"/>
+      <x:c r="BP12"/>
+      <x:c r="BQ12"/>
+      <x:c r="BR12"/>
+      <x:c r="BS12"/>
+      <x:c r="BT12"/>
+      <x:c r="BU12"/>
+      <x:c r="BV12"/>
+      <x:c r="BW12"/>
+      <x:c r="BX12"/>
+      <x:c r="BY12"/>
+      <x:c r="BZ12"/>
+      <x:c r="CA12"/>
+      <x:c r="CB12"/>
+      <x:c r="CC12"/>
+      <x:c r="CD12"/>
+      <x:c r="CE12"/>
+      <x:c r="CF12"/>
+      <x:c r="CG12"/>
+      <x:c r="CH12"/>
+      <x:c r="CI12"/>
+      <x:c r="CJ12"/>
+      <x:c r="CK12"/>
+      <x:c r="CL12"/>
+      <x:c r="CM12" t="str">
+        <x:v>Source: Portfolio - Tianyi WANG - 20 mb.pdf, PDF page 17. Website models and images await author delivery.</x:v>
+      </x:c>
+      <x:c r="CN12"/>
+      <x:c r="CO12"/>
+      <x:c r="CP12"/>
+      <x:c r="CQ12"/>
+      <x:c r="CR12" t="str">
+        <x:v>2026-09-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>project</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>storyline-studio</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>Storyline Studio</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>Storyline Studio</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>Storyline Studio</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>Storyline Studio</x:v>
+      </x:c>
+      <x:c r="I13"/>
+      <x:c r="J13"/>
+      <x:c r="K13" t="str">
+        <x:v>A mid-rise film studio translating parallel cinematic timelines into spatial organization, testing the relationship between narrow circulation spaces and larger rooms for collective activity.</x:v>
+      </x:c>
+      <x:c r="L13" t="str">
+        <x:v>将电影中平行时间线的叙事转译为空间组织，研究狭长动线与集体活动大空间之间关系的中层电影工作室设计。</x:v>
+      </x:c>
+      <x:c r="M13"/>
+      <x:c r="N13"/>
+      <x:c r="O13"/>
+      <x:c r="P13"/>
+      <x:c r="Q13" t="str">
+        <x:v>Tianyi WANG</x:v>
+      </x:c>
+      <x:c r="R13" t="str">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="S13"/>
+      <x:c r="T13"/>
+      <x:c r="U13"/>
+      <x:c r="V13"/>
+      <x:c r="W13"/>
+      <x:c r="X13"/>
+      <x:c r="Y13"/>
+      <x:c r="Z13"/>
+      <x:c r="AA13"/>
+      <x:c r="AB13"/>
+      <x:c r="AC13"/>
+      <x:c r="AD13"/>
+      <x:c r="AE13"/>
+      <x:c r="AF13" t="str">
+        <x:v>2019 · Manhattan, New York</x:v>
+      </x:c>
+      <x:c r="AG13" t="str">
+        <x:v>2019 · Pratt ARCH 202 · Individual work</x:v>
+      </x:c>
+      <x:c r="AH13" t="str">
+        <x:v>2019 · Pratt ARCH 202 · 个人作品</x:v>
+      </x:c>
+      <x:c r="AI13" t="str">
+        <x:v>Study</x:v>
+      </x:c>
+      <x:c r="AJ13" t="str">
+        <x:v>stage-student</x:v>
+      </x:c>
+      <x:c r="AK13" t="str">
+        <x:v>Education</x:v>
+      </x:c>
+      <x:c r="AL13" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="AM13" t="str">
+        <x:v>Text study</x:v>
+      </x:c>
+      <x:c r="AN13" t="str">
+        <x:v>文字研究</x:v>
+      </x:c>
+      <x:c r="AO13" t="str">
+        <x:v>A mid-rise film studio translating parallel cinematic timelines into spatial organization, testing the relationship between narrow circulation spaces and larger rooms for collective activity.</x:v>
+      </x:c>
+      <x:c r="AP13" t="str">
+        <x:v>将电影中平行时间线的叙事转译为空间组织，研究狭长动线与集体活动大空间之间关系的中层电影工作室设计。</x:v>
+      </x:c>
+      <x:c r="AQ13" t="str">
+        <x:v>Pratt ARCH 202 · Individual work. Site: Manhattan, New York. Credits: Tianyi WANG.</x:v>
+      </x:c>
+      <x:c r="AR13" t="str">
+        <x:v>Pratt ARCH 202 · 个人作品。项目地点：纽约曼哈顿。作者：Tianyi WANG。</x:v>
+      </x:c>
+      <x:c r="AS13" t="str">
+        <x:v>Pratt ARCH 202 · Individual work</x:v>
+      </x:c>
+      <x:c r="AT13" t="str">
+        <x:v>Pratt ARCH 202 · 个人作品</x:v>
+      </x:c>
+      <x:c r="AU13" t="str">
+        <x:v>Site: Manhattan, New York</x:v>
+      </x:c>
+      <x:c r="AV13" t="str">
+        <x:v>项目地点：纽约曼哈顿</x:v>
+      </x:c>
+      <x:c r="AW13" t="str">
+        <x:v>Academic design proposal.</x:v>
+      </x:c>
+      <x:c r="AX13" t="str">
+        <x:v>学术设计方案。</x:v>
+      </x:c>
+      <x:c r="AY13"/>
+      <x:c r="AZ13"/>
+      <x:c r="BA13"/>
+      <x:c r="BB13"/>
+      <x:c r="BC13"/>
+      <x:c r="BD13"/>
+      <x:c r="BE13"/>
+      <x:c r="BF13"/>
+      <x:c r="BG13"/>
+      <x:c r="BH13"/>
+      <x:c r="BI13"/>
+      <x:c r="BJ13"/>
+      <x:c r="BK13"/>
+      <x:c r="BL13"/>
+      <x:c r="BM13"/>
+      <x:c r="BN13"/>
+      <x:c r="BO13"/>
+      <x:c r="BP13"/>
+      <x:c r="BQ13"/>
+      <x:c r="BR13"/>
+      <x:c r="BS13"/>
+      <x:c r="BT13"/>
+      <x:c r="BU13"/>
+      <x:c r="BV13"/>
+      <x:c r="BW13"/>
+      <x:c r="BX13"/>
+      <x:c r="BY13"/>
+      <x:c r="BZ13"/>
+      <x:c r="CA13"/>
+      <x:c r="CB13"/>
+      <x:c r="CC13"/>
+      <x:c r="CD13"/>
+      <x:c r="CE13"/>
+      <x:c r="CF13"/>
+      <x:c r="CG13"/>
+      <x:c r="CH13"/>
+      <x:c r="CI13"/>
+      <x:c r="CJ13"/>
+      <x:c r="CK13"/>
+      <x:c r="CL13"/>
+      <x:c r="CM13" t="str">
+        <x:v>Source: Portfolio - Tianyi WANG - 20 mb.pdf, PDF page 9. Website models and images await author delivery.</x:v>
+      </x:c>
+      <x:c r="CN13"/>
+      <x:c r="CO13"/>
+      <x:c r="CP13"/>
+      <x:c r="CQ13"/>
+      <x:c r="CR13" t="str">
+        <x:v>2026-09-08</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1988,7 +2982,7 @@
         <x:v>project-03</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D2" t="str">
         <x:v>50</x:v>
@@ -2136,7 +3130,7 @@
         <x:v>project-04</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D3" t="str">
         <x:v>60</x:v>
@@ -2290,20 +3284,20 @@
         <x:v>1110</x:v>
       </x:c>
       <x:c r="E4" t="str">
-        <x:v>Architecture</x:v>
+        <x:v>Professional practice</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>Architecture</x:v>
+        <x:v>职业实践</x:v>
       </x:c>
       <x:c r="G4" t="str"/>
       <x:c r="H4" t="str"/>
       <x:c r="I4" t="str"/>
       <x:c r="J4" t="str"/>
       <x:c r="K4" t="str">
-        <x:v>Three years in professional practice brought spatial ideas into collaboration, delivery, constraints, and presentation discipline.</x:v>
+        <x:v>Architectural Designer and AIGC Lead, connecting concept development, visualization and repeatable AI production workflows.</x:v>
       </x:c>
       <x:c r="L4" t="str">
-        <x:v>三年的建筑职业阶段让空间想法进入真实协作、交付和限制条件中；这里强调的是专业判断、表达能力和项目推进方式。</x:v>
+        <x:v>作为建筑设计师与 AIGC 负责人，将概念设计、视觉表达与可复用的 AI 制作流程连接起来。</x:v>
       </x:c>
       <x:c r="M4" t="str"/>
       <x:c r="N4" t="str"/>
@@ -2377,36 +3371,34 @@
       <x:c r="BR4" t="str"/>
       <x:c r="BS4" t="str"/>
       <x:c r="BT4" t="str">
-        <x:v>Three-year professional stage</x:v>
+        <x:v>Aedas · Shenzhen · September 2023–present</x:v>
       </x:c>
       <x:c r="BU4" t="str">
-        <x:v>Three-year professional stage</x:v>
+        <x:v>Aedas · 深圳 · 2023 年 9 月至今</x:v>
       </x:c>
       <x:c r="BV4" t="str">
-        <x:v>Worked across concept design, modeling, drawings, visualization, material research, and presentation packages.
-Kept spatial narrative and representation standards clear across changing project types, scales, and phases.
-Use anonymized diagrams, abstracted models, and process notes for confidential work, preserving the professional logic without exposing restricted material.</x:v>
+        <x:v>Led the in-house AIGC team and built AI rendering and animation workflows with Stable Diffusion WebUI and ComfyUI, later extending to Lovart.
+Developed reusable prompt templates and workflows; produced renders, AI animation and video for more than 20 projects.
+Collaborated on concepts, 3D modeling, post-production and presentations; promoted from Junior Designer to Designer in early 2025.</x:v>
       </x:c>
       <x:c r="BW4" t="str">
-        <x:v>参与概念设计、建模、图纸、渲染、材料研究和汇报材料组织。
-在项目类型、尺度和阶段变化中保持清晰的空间叙事与表达标准。
-对保密项目采用脱敏 diagram、抽象模型和过程说明，保留专业脉络而不暴露敏感资料。</x:v>
+        <x:v>带领内部 AIGC 团队，以 Stable Diffusion WebUI、ComfyUI 建立 AI 渲染与动画流程，之后扩展至 Lovart。
+开发可复用的提示词模板和工作流程，为 20 多个项目制作渲染、AI 动画与视频。
+参与概念设计、三维建模、后期和汇报；2025 年初由 Junior Designer 晋升为 Designer。</x:v>
       </x:c>
       <x:c r="BX4" t="str">
-        <x:v>Professional projects can become a corridor organized by project phase and role.
-Public material can show images, models, detail fragments, and concise responsibility notes.
-Restricted material can appear as abstract spatial slices, explaining working methods rather than showing confidential drawings.</x:v>
+        <x:v>2025–2026 · UABB Huaqiangbei study: visual narratives and models examining urban history and possible future city scenarios.
+April 2025 · Game Jam · Lead level design for an in-game city, using urban fabric to organize the environment.</x:v>
       </x:c>
       <x:c r="BY4" t="str">
-        <x:v>职业项目会被整理成一条空间走廊，按项目阶段和参与角色组织。
-公开素材会展示图像、模型、局部细节和简短职责说明。
-非公开素材会以抽象空间切片呈现，让访问者理解工作方式而不是浏览机密图纸。</x:v>
+        <x:v>2025–2026 · UABB 华强北研究：通过视觉叙事与模型呈现城市历史及未来城市情境。
+2025 年 4 月 · Game Jam · 主导游戏城市关卡设计，以城市肌理组织场景。</x:v>
       </x:c>
       <x:c r="BZ4" t="str">
-        <x:v>In SPACE, this can become a professional corridor where each architecture project is an exhibit node; confidential projects stay abstract.</x:v>
+        <x:v>Concepts, models and images are developed together to make spatial decisions clear across a team.</x:v>
       </x:c>
       <x:c r="CA4" t="str">
-        <x:v>SPACE 中可以做成一条职业走廊，每个建筑项目是一个展品节点，保密项目用抽象信息呈现。</x:v>
+        <x:v>将概念、模型与图像共同推进，使空间判断能在团队协作中清楚传达。</x:v>
       </x:c>
       <x:c r="CB4" t="str"/>
       <x:c r="CC4" t="str"/>
@@ -3758,7 +4750,7 @@
         <x:v>project-05</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D2" t="str">
         <x:v>70</x:v>
@@ -3906,7 +4898,7 @@
         <x:v>project-06</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D3" t="str">
         <x:v>80</x:v>
@@ -4054,7 +5046,7 @@
         <x:v>project-07</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D4" t="str">
         <x:v>90</x:v>
@@ -4202,7 +5194,7 @@
         <x:v>project-08</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>100</x:v>
@@ -4356,36 +5348,30 @@
         <x:v>1000</x:v>
       </x:c>
       <x:c r="E6" t="str">
-        <x:v>LizzardKevin</x:v>
+        <x:v>Tianyi WANG / LizzardKevin</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>LizzardKevin</x:v>
+        <x:v>王天奕 / LizzardKevin</x:v>
       </x:c>
       <x:c r="G6" t="str"/>
       <x:c r="H6" t="str"/>
       <x:c r="I6" t="str"/>
       <x:c r="J6" t="str"/>
       <x:c r="K6" t="str">
-        <x:v>I keep architecture training, spatial narrative, photography, band memory, and AI image workflows in the same personal archive. SPACE carries the more immersive exhibits; this page stays closer to a readable profile so visitors can quickly understand who I am, what I have done, and where the archive can grow next.</x:v>
+        <x:v>I am Tianyi WANG / LizzardKevin, a Shenzhen-based architectural designer and AIGC visual creator. My work connects architectural training at Pratt and Columbia with spatial storytelling, visualization and AI production workflows at Aedas.</x:v>
       </x:c>
       <x:c r="L6" t="str">
-        <x:v>我把建筑训练、空间叙事、摄影观察、乐队经验和 AI 创作方法放在同一个个人档案里。SPACE 会承载更沉浸的展品与作品，而这里保持更传统的简历状态，方便快速理解我是谁、做过什么、还能继续展开什么。</x:v>
+        <x:v>我是王天奕 / LizzardKevin，现居深圳，从事建筑设计与 AIGC 视觉创作。从 Pratt、Columbia 的建筑训练到 Aedas 的职业实践，我关注如何用空间叙事、图像和 AI 工作流程表达设计。</x:v>
       </x:c>
       <x:c r="M6" t="str"/>
       <x:c r="N6" t="str"/>
       <x:c r="O6" t="str">
-        <x:v>AI visual creator
-spatial designer
-photographer
-bassist
-etc.</x:v>
+        <x:v>Architectural designer
+AIGC visual creator</x:v>
       </x:c>
       <x:c r="P6" t="str">
-        <x:v>AI 创意设计师
-空间设计师
-摄影师
-贝斯手
-etc.</x:v>
+        <x:v>建筑设计师
+AIGC 视觉创作者</x:v>
       </x:c>
       <x:c r="Q6" t="str"/>
       <x:c r="R6" t="str"/>
@@ -4397,10 +5383,10 @@
       <x:c r="X6" t="str"/>
       <x:c r="Y6" t="str"/>
       <x:c r="Z6" t="str">
-        <x:v>Architecture, creative technology, image-making, music, and personal culture archive.</x:v>
+        <x:v>Aedas · Architectural Designer / AIGC Lead · since September 2023</x:v>
       </x:c>
       <x:c r="AA6" t="str">
-        <x:v>Architecture, creative technology, image-making, music, and personal culture archive.</x:v>
+        <x:v>Aedas · 建筑设计师 / AIGC 负责人 · 2023 年 9 月起</x:v>
       </x:c>
       <x:c r="AB6" t="str"/>
       <x:c r="AC6" t="str"/>
@@ -4463,7 +5449,7 @@
       <x:c r="CH6" t="str"/>
       <x:c r="CI6" t="str"/>
       <x:c r="CJ6" t="str">
-        <x:v>New York / Shanghai</x:v>
+        <x:v>Shenzhen / 深圳</x:v>
       </x:c>
       <x:c r="CK6" t="str"/>
       <x:c r="CL6" t="str"/>
@@ -4488,10 +5474,10 @@
         <x:v>1010</x:v>
       </x:c>
       <x:c r="E7" t="str">
-        <x:v>Contact</x:v>
+        <x:v>Email</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>Contact</x:v>
+        <x:v>邮箱</x:v>
       </x:c>
       <x:c r="G7" t="str"/>
       <x:c r="H7" t="str"/>
@@ -4573,12 +5559,14 @@
       <x:c r="CF7" t="str"/>
       <x:c r="CG7" t="str"/>
       <x:c r="CH7" t="str">
-        <x:v>Open for selected collaborations</x:v>
+        <x:v>lizzardkevin@gmail.com</x:v>
       </x:c>
       <x:c r="CI7" t="str">
-        <x:v>Open for selected collaborations</x:v>
-      </x:c>
-      <x:c r="CJ7" t="str"/>
+        <x:v>lizzardkevin@gmail.com</x:v>
+      </x:c>
+      <x:c r="CJ7" t="str">
+        <x:v>mailto:lizzardkevin@gmail.com</x:v>
+      </x:c>
       <x:c r="CK7" t="str"/>
       <x:c r="CL7" t="str"/>
       <x:c r="CM7" t="str"/>
@@ -4602,10 +5590,10 @@
         <x:v>1020</x:v>
       </x:c>
       <x:c r="E8" t="str">
-        <x:v>Location</x:v>
+        <x:v>Email</x:v>
       </x:c>
       <x:c r="F8" t="str">
-        <x:v>Location</x:v>
+        <x:v>邮箱</x:v>
       </x:c>
       <x:c r="G8" t="str"/>
       <x:c r="H8" t="str"/>
@@ -4687,12 +5675,14 @@
       <x:c r="CF8" t="str"/>
       <x:c r="CG8" t="str"/>
       <x:c r="CH8" t="str">
-        <x:v>New York / Shanghai</x:v>
+        <x:v>lizzardkevin@qq.com</x:v>
       </x:c>
       <x:c r="CI8" t="str">
-        <x:v>New York / Shanghai</x:v>
-      </x:c>
-      <x:c r="CJ8" t="str"/>
+        <x:v>lizzardkevin@qq.com</x:v>
+      </x:c>
+      <x:c r="CJ8" t="str">
+        <x:v>mailto:lizzardkevin@qq.com</x:v>
+      </x:c>
       <x:c r="CK8" t="str"/>
       <x:c r="CL8" t="str"/>
       <x:c r="CM8" t="str"/>
@@ -4832,10 +5822,10 @@
         <x:v>1040</x:v>
       </x:c>
       <x:c r="E10" t="str">
-        <x:v>Practice</x:v>
+        <x:v>Based in</x:v>
       </x:c>
       <x:c r="F10" t="str">
-        <x:v>Practice</x:v>
+        <x:v>现居</x:v>
       </x:c>
       <x:c r="G10" t="str"/>
       <x:c r="H10" t="str"/>
@@ -4917,10 +5907,10 @@
       <x:c r="CF10" t="str"/>
       <x:c r="CG10" t="str"/>
       <x:c r="CH10" t="str">
-        <x:v>Architecture + creative technology</x:v>
+        <x:v>Shenzhen / 深圳</x:v>
       </x:c>
       <x:c r="CI10" t="str">
-        <x:v>Architecture + creative technology</x:v>
+        <x:v>Shenzhen / 深圳</x:v>
       </x:c>
       <x:c r="CJ10" t="str"/>
       <x:c r="CK10" t="str"/>
@@ -4946,10 +5936,10 @@
         <x:v>1050</x:v>
       </x:c>
       <x:c r="E11" t="str">
-        <x:v>Archive</x:v>
+        <x:v>Phone</x:v>
       </x:c>
       <x:c r="F11" t="str">
-        <x:v>Archive</x:v>
+        <x:v>电话</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11" t="str"/>
@@ -5031,12 +6021,14 @@
       <x:c r="CF11" t="str"/>
       <x:c r="CG11" t="str"/>
       <x:c r="CH11" t="str">
-        <x:v>Interactive SPACE in progress</x:v>
+        <x:v>+86 13682600019</x:v>
       </x:c>
       <x:c r="CI11" t="str">
-        <x:v>Interactive SPACE in progress</x:v>
-      </x:c>
-      <x:c r="CJ11" t="str"/>
+        <x:v>+86 13682600019</x:v>
+      </x:c>
+      <x:c r="CJ11" t="str">
+        <x:v>tel:+8613682600019</x:v>
+      </x:c>
       <x:c r="CK11" t="str"/>
       <x:c r="CL11" t="str"/>
       <x:c r="CM11" t="str"/>
@@ -5054,7 +6046,7 @@
         <x:v>profile_link_06</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D12" t="str">
         <x:v>1060</x:v>
@@ -5177,17 +6169,17 @@
         <x:v>Photography</x:v>
       </x:c>
       <x:c r="F13" t="str">
-        <x:v>Photography</x:v>
+        <x:v>摄影</x:v>
       </x:c>
       <x:c r="G13" t="str"/>
       <x:c r="H13" t="str"/>
       <x:c r="I13" t="str"/>
       <x:c r="J13" t="str"/>
       <x:c r="K13" t="str">
-        <x:v>Photography is how I practice observation: cities, light, people, speed, and chance feed back into spatial design and AI image work.</x:v>
+        <x:v>Photography informs how I notice light, scale and everyday spaces.</x:v>
       </x:c>
       <x:c r="L13" t="str">
-        <x:v>摄影是我训练观察的方式：城市、光线、人物、速度和偶然性会反过来影响空间设计与 AI 视觉创作。</x:v>
+        <x:v>摄影影响我对光线、尺度和日常空间的观察。</x:v>
       </x:c>
       <x:c r="M13" t="str"/>
       <x:c r="N13" t="str"/>
@@ -5261,36 +6253,20 @@
       <x:c r="BR13" t="str"/>
       <x:c r="BS13" t="str"/>
       <x:c r="BT13" t="str">
-        <x:v>Image-making and spatial observation</x:v>
+        <x:v>Urban observation</x:v>
       </x:c>
       <x:c r="BU13" t="str">
-        <x:v>Image-making and spatial observation</x:v>
-      </x:c>
-      <x:c r="BV13" t="str">
-        <x:v>Look for atmosphere in architecture, streets, night scenes, live shows, and travel fragments.
-Organize images as series, so photography becomes an ongoing observation archive rather than a set of isolated portfolio shots.
-Translate composition, contrast, and color habits from photography into the WebGPU gallery and AI image experiments.</x:v>
-      </x:c>
-      <x:c r="BW13" t="str">
-        <x:v>关注建筑、街头、夜景、演出现场和旅行切片中的空间气氛。
-用系列化方式整理图像，让照片不只是单张漂亮画面，而是持续的观察档案。
-把摄影中的构图、光比和色彩经验转译到 WebGPU 展厅和 AI 图像实验里。</x:v>
-      </x:c>
-      <x:c r="BX13" t="str">
-        <x:v>Photo walls can unfold by series, each with place, time, and a short statement.
-The image room should feel closer to a darkroom or city fragment than a generic album grid.
-Public images can connect outward; private images can appear only as curated fragments inside SPACE.</x:v>
-      </x:c>
-      <x:c r="BY13" t="str">
-        <x:v>照片墙会以系列为单位展开，每组照片保留地点、时间和简短 statement。
-影像展区会更像暗房或城市切片，而不是普通相册网格。
-可公开图像会连接到外部发布渠道，未公开图像只在 SPACE 中以策展方式出现。</x:v>
-      </x:c>
+        <x:v>城市观察</x:v>
+      </x:c>
+      <x:c r="BV13" t="str"/>
+      <x:c r="BW13" t="str"/>
+      <x:c r="BX13" t="str"/>
+      <x:c r="BY13" t="str"/>
       <x:c r="BZ13" t="str">
-        <x:v>In SPACE, this can become a photo wall, darkroom, or city-slice zone where images stand as their own exhibit area.</x:v>
+        <x:v>Photography informs how I notice light, scale and everyday spaces.</x:v>
       </x:c>
       <x:c r="CA13" t="str">
-        <x:v>SPACE 中可以做成照片墙、暗房或城市切片区域，让影像成为独立展区。</x:v>
+        <x:v>摄影影响我对光线、尺度和日常空间的观察。</x:v>
       </x:c>
       <x:c r="CB13" t="str"/>
       <x:c r="CC13" t="str"/>
@@ -5327,17 +6303,17 @@
         <x:v>Music / Band</x:v>
       </x:c>
       <x:c r="F14" t="str">
-        <x:v>Music / Band</x:v>
+        <x:v>音乐 / 乐队</x:v>
       </x:c>
       <x:c r="G14" t="str"/>
       <x:c r="H14" t="str"/>
       <x:c r="I14" t="str"/>
       <x:c r="J14" t="str"/>
       <x:c r="K14" t="str">
-        <x:v>Bass and band memory bring sound, low frequency, and a live-room feeling into the archive; they are also the most natural source for SPACE audio exhibits.</x:v>
+        <x:v>Bass and band practice are part of my life beyond architectural work.</x:v>
       </x:c>
       <x:c r="L14" t="str">
-        <x:v>贝斯和乐队经验给这个个人档案带来声音、低频和现场感；它也是 SPACE 音频展品系统最自然的内容来源。</x:v>
+        <x:v>建筑工作之外，贝斯与乐队练习也是我的生活的一部分。</x:v>
       </x:c>
       <x:c r="M14" t="str"/>
       <x:c r="N14" t="str"/>
@@ -5411,36 +6387,20 @@
       <x:c r="BR14" t="str"/>
       <x:c r="BS14" t="str"/>
       <x:c r="BT14" t="str">
-        <x:v>Bass, rehearsal, live performance</x:v>
+        <x:v>Bass and rhythm</x:v>
       </x:c>
       <x:c r="BU14" t="str">
-        <x:v>Bass, rehearsal, live performance</x:v>
-      </x:c>
-      <x:c r="BV14" t="str">
-        <x:v>Draw a sonic identity from rehearsals, demos, live recordings, and performance photos.
-Care about how bass lines support rhythm, space, and stage atmosphere, not only gear lists.
-Connect audio playback, progress bars, and Focus exhibits so work can be heard and viewed at the same time.</x:v>
-      </x:c>
-      <x:c r="BW14" t="str">
-        <x:v>从排练、demo、live recording 和演出照片中提取声音身份。
-关注贝斯线如何支撑节奏、空间和舞台氛围，而不只展示器材清单。
-把音频播放、进度条和 Focus 展品连接起来，让作品可以被听见也可以被观看。</x:v>
-      </x:c>
-      <x:c r="BX14" t="str">
-        <x:v>The music area can feel like a rehearsal corner, holding instruments, posters, and audio fragments.
-Playable exhibits can connect demos, live clips, or low-frequency loops.
-Each sound node should keep simple context: scene, track state, role, and recording time.</x:v>
-      </x:c>
-      <x:c r="BY14" t="str">
-        <x:v>音乐区域会以 rehearsal corner 的方式呈现，保留器材、海报和声音片段。
-可播放展品会连接 demo、live clip 或低频 loop。
-每个声音节点会保留简单背景：场景、曲目状态、参与角色和记录时间。</x:v>
-      </x:c>
+        <x:v>贝斯与节奏</x:v>
+      </x:c>
+      <x:c r="BV14" t="str"/>
+      <x:c r="BW14" t="str"/>
+      <x:c r="BX14" t="str"/>
+      <x:c r="BY14" t="str"/>
       <x:c r="BZ14" t="str">
-        <x:v>In SPACE, this can become a rehearsal corner or sound exhibit where clicking plays a demo, live clip, or bass line.</x:v>
+        <x:v>Bass and band practice are part of my life beyond architectural work.</x:v>
       </x:c>
       <x:c r="CA14" t="str">
-        <x:v>SPACE 中可以做成 rehearsal corner 或声音展品，点击后播放 demo、live clip 或 bass line。</x:v>
+        <x:v>建筑工作之外，贝斯与乐队练习也是我的生活的一部分。</x:v>
       </x:c>
       <x:c r="CB14" t="str"/>
       <x:c r="CC14" t="str"/>
@@ -5474,20 +6434,20 @@
         <x:v>1140</x:v>
       </x:c>
       <x:c r="E15" t="str">
-        <x:v>Anime / Culture</x:v>
+        <x:v>Visual culture</x:v>
       </x:c>
       <x:c r="F15" t="str">
-        <x:v>Anime / Culture</x:v>
+        <x:v>视觉文化</x:v>
       </x:c>
       <x:c r="G15" t="str"/>
       <x:c r="H15" t="str"/>
       <x:c r="I15" t="str"/>
       <x:c r="J15" t="str"/>
       <x:c r="K15" t="str">
-        <x:v>Personal culture enters the archive as aesthetic source and narrative influence, not as a pile of titles; the point is how it changes my spatial, color, and character imagination.</x:v>
+        <x:v>Animation, games and visual references inform my interest in atmosphere and narrative.</x:v>
       </x:c>
       <x:c r="L15" t="str">
-        <x:v>个人文化影响会以审美来源和叙事影响的方式进入档案，而不是直接堆作品名；重点是它们如何改变我的空间、色彩和角色想象。</x:v>
+        <x:v>动画、游戏与视觉参考影响我对气氛和叙事的兴趣。</x:v>
       </x:c>
       <x:c r="M15" t="str"/>
       <x:c r="N15" t="str"/>
@@ -5561,36 +6521,20 @@
       <x:c r="BR15" t="str"/>
       <x:c r="BS15" t="str"/>
       <x:c r="BT15" t="str">
-        <x:v>Personal references and visual influence</x:v>
+        <x:v>Animation and games</x:v>
       </x:c>
       <x:c r="BU15" t="str">
-        <x:v>Personal references and visual influence</x:v>
-      </x:c>
-      <x:c r="BV15" t="str">
-        <x:v>Organize animation, manga, games, visual novels, and music projects as personal sources of taste.
-Prioritize original, inspired-by, or experimental work instead of directly reposting official images.
-Track how color, character atmosphere, spatial narrative, and music emotion migrate between media.</x:v>
-      </x:c>
-      <x:c r="BW15" t="str">
-        <x:v>把动画、漫画、游戏、视觉小说和音乐企划作为个人审美来源来整理。
-优先展示原创、inspired-by 或实验性作品，避免直接搬运未经授权的官方图像。
-关注色彩、角色气质、空间叙事和音乐情绪如何在不同媒介之间迁移。</x:v>
-      </x:c>
-      <x:c r="BX15" t="str">
-        <x:v>The culture area can behave like a reference archive with original images, posters, AI tests, and text notes.
-Each node explains where an influence comes from and how it enters space, image, or sound work.
-Public presentation should foreground original output; references stay mostly as textual clues.</x:v>
-      </x:c>
-      <x:c r="BY15" t="str">
-        <x:v>文化影响区会更像 reference archive，展示原创图像、poster、AI 实验和文字说明。
-每个节点解释影响来自哪里，以及它如何进入空间、影像或声音创作。
-公开呈现以原创内容为主，引用内容只作为文本层面的线索。</x:v>
-      </x:c>
+        <x:v>动画与游戏</x:v>
+      </x:c>
+      <x:c r="BV15" t="str"/>
+      <x:c r="BW15" t="str"/>
+      <x:c r="BX15" t="str"/>
+      <x:c r="BY15" t="str"/>
       <x:c r="BZ15" t="str">
-        <x:v>In SPACE, this can become a cultural influence archive for original work and inspiration notes, not a direct repost wall.</x:v>
+        <x:v>Animation, games and visual references inform my interest in atmosphere and narrative.</x:v>
       </x:c>
       <x:c r="CA15" t="str">
-        <x:v>SPACE 中可以做成文化影响档案区，展示原创内容和灵感说明，而不是直接搬运官方素材。</x:v>
+        <x:v>动画、游戏与视觉参考影响我对气氛和叙事的兴趣。</x:v>
       </x:c>
       <x:c r="CB15" t="str"/>
       <x:c r="CC15" t="str"/>
@@ -6258,7 +7202,7 @@
         <x:v>project-09</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D2" t="str">
         <x:v>110</x:v>
@@ -6406,7 +7350,7 @@
         <x:v>project-10</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D3" t="str">
         <x:v>120</x:v>
@@ -6554,7 +7498,7 @@
         <x:v>project-11</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D4" t="str">
         <x:v>130</x:v>
@@ -6708,20 +7652,20 @@
         <x:v>1150</x:v>
       </x:c>
       <x:c r="E5" t="str">
-        <x:v>Other / Experiments</x:v>
+        <x:v>Experiments</x:v>
       </x:c>
       <x:c r="F5" t="str">
-        <x:v>Other / Experiments</x:v>
+        <x:v>实验</x:v>
       </x:c>
       <x:c r="G5" t="str"/>
       <x:c r="H5" t="str"/>
       <x:c r="I5" t="str"/>
       <x:c r="J5" t="str"/>
       <x:c r="K5" t="str">
-        <x:v>This area holds AI, WebGPU, writing, and experiments that do not fit a single category yet; it is the lab where SPACE keeps growing.</x:v>
+        <x:v>I explore how spatial ideas can become interactive environments and repeatable visual workflows.</x:v>
       </x:c>
       <x:c r="L5" t="str">
-        <x:v>这一段收纳 AI、WebGPU、写作和其他暂时无法归类的实验；它是 SPACE 持续生长的实验室。</x:v>
+        <x:v>我探索空间想法如何转化为交互环境，以及可复用的视觉工作流程。</x:v>
       </x:c>
       <x:c r="M5" t="str"/>
       <x:c r="N5" t="str"/>
@@ -6795,36 +7739,20 @@
       <x:c r="BR5" t="str"/>
       <x:c r="BS5" t="str"/>
       <x:c r="BT5" t="str">
-        <x:v>AI, web, writing, and future work</x:v>
+        <x:v>SPACE and AI workflows</x:v>
       </x:c>
       <x:c r="BU5" t="str">
-        <x:v>AI, web, writing, and future work</x:v>
-      </x:c>
-      <x:c r="BV5" t="str">
-        <x:v>Collect AI image and video work, spatial concept generation, prompt design, and workflow research.
-Treat Three.js, WebGPU, and interactive portfolio work as real creative media, not just technical demos.
-Keep essays, devlogs, research notes, and failed tests visible, so process becomes part of the archive.</x:v>
-      </x:c>
-      <x:c r="BW5" t="str">
-        <x:v>整理 AI 图像、视频、空间概念生成、prompt design 和 workflow 研究。
-把 Three.js、WebGPU 和 interactive portfolio 当作真实作品载体，而不是技术 demo。
-保留 essay、devlog、研究笔记和实验失败记录，让过程本身成为档案的一部分。</x:v>
-      </x:c>
-      <x:c r="BX5" t="str">
-        <x:v>The lab area can keep gaining exhibits: generated results, process screenshots, and design notes.
-DevStories becomes the technical narrative layer, explaining how each build round changes SPACE.
-Collaboration directions can orbit creative technology, spatial design, image-making, exhibition, music, and AI workflow.</x:v>
-      </x:c>
-      <x:c r="BY5" t="str">
-        <x:v>实验室区域会持续追加新展品，包含生成结果、过程截图和设计说明。
-DevStories 会成为技术叙事层，解释每轮构建如何改变 SPACE。
-合作方向会围绕创意技术、空间设计、影像、展览、音乐和 AI workflow 展开。</x:v>
-      </x:c>
+        <x:v>SPACE 与 AI 工作流程</x:v>
+      </x:c>
+      <x:c r="BV5" t="str"/>
+      <x:c r="BW5" t="str"/>
+      <x:c r="BX5" t="str"/>
+      <x:c r="BY5" t="str"/>
       <x:c r="BZ5" t="str">
-        <x:v>In SPACE, this can stay as a living lab where future work expands directly into new exhibit nodes.</x:v>
+        <x:v>I explore how spatial ideas can become interactive environments and repeatable visual workflows.</x:v>
       </x:c>
       <x:c r="CA5" t="str">
-        <x:v>SPACE 中可以作为持续更新的实验室区域，后续新内容直接扩展为新的展品节点。</x:v>
+        <x:v>我探索空间想法如何转化为交互环境，以及可复用的视觉工作流程。</x:v>
       </x:c>
       <x:c r="CB5" t="str"/>
       <x:c r="CC5" t="str"/>
@@ -20929,10 +21857,10 @@
         <x:v>projectDetails.currentSignal</x:v>
       </x:c>
       <x:c r="CH127" t="str">
-        <x:v>Current Signal</x:v>
+        <x:v>Role / Context</x:v>
       </x:c>
       <x:c r="CI127" t="str">
-        <x:v>当前信号</x:v>
+        <x:v>角色 / 背景</x:v>
       </x:c>
       <x:c r="CJ127" t="str"/>
       <x:c r="CK127" t="str"/>
@@ -21043,10 +21971,10 @@
         <x:v>projectDetails.spaceLayer</x:v>
       </x:c>
       <x:c r="CH128" t="str">
-        <x:v>SPACE Layer</x:v>
+        <x:v>Project context</x:v>
       </x:c>
       <x:c r="CI128" t="str">
-        <x:v>SPACE 层级</x:v>
+        <x:v>项目语境</x:v>
       </x:c>
       <x:c r="CJ128" t="str"/>
       <x:c r="CK128" t="str"/>
@@ -21157,10 +22085,10 @@
         <x:v>projectDetails.archiveNote</x:v>
       </x:c>
       <x:c r="CH129" t="str">
-        <x:v>Archive Note</x:v>
+        <x:v>Project status</x:v>
       </x:c>
       <x:c r="CI129" t="str">
-        <x:v>档案备注</x:v>
+        <x:v>项目属性</x:v>
       </x:c>
       <x:c r="CJ129" t="str"/>
       <x:c r="CK129" t="str"/>
@@ -21727,10 +22655,10 @@
         <x:v>projects.lede</x:v>
       </x:c>
       <x:c r="CH134" t="str">
-        <x:v>A phone-readable index for future exhibition rooms. Project details stay text-first until real media is ready.</x:v>
+        <x:v>Selected architectural work and academic design studies.</x:v>
       </x:c>
       <x:c r="CI134" t="str">
-        <x:v>适合手机快速阅读的展厅索引。真实媒体完成前，项目详情先保持文字优先。</x:v>
+        <x:v>建筑作品与学术设计研究。</x:v>
       </x:c>
       <x:c r="CJ134" t="str"/>
       <x:c r="CK134" t="str"/>
@@ -22092,7 +23020,7 @@
         <x:v>mobile_terminal_soul_bio</x:v>
       </x:c>
       <x:c r="C138" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D138" t="str">
         <x:v>5025</x:v>
@@ -22206,7 +23134,7 @@
         <x:v>mobile_terminal_soul_sections_0_title</x:v>
       </x:c>
       <x:c r="C139" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D139" t="str">
         <x:v>5026</x:v>
@@ -22320,7 +23248,7 @@
         <x:v>mobile_terminal_soul_sections_0_meta</x:v>
       </x:c>
       <x:c r="C140" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D140" t="str">
         <x:v>5027</x:v>
@@ -22434,7 +23362,7 @@
         <x:v>mobile_terminal_soul_sections_0_summary</x:v>
       </x:c>
       <x:c r="C141" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D141" t="str">
         <x:v>5028</x:v>
@@ -22548,7 +23476,7 @@
         <x:v>mobile_terminal_soul_sections_0_details_0</x:v>
       </x:c>
       <x:c r="C142" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D142" t="str">
         <x:v>5029</x:v>
@@ -22662,7 +23590,7 @@
         <x:v>mobile_terminal_soul_sections_0_details_1</x:v>
       </x:c>
       <x:c r="C143" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D143" t="str">
         <x:v>5030</x:v>
@@ -22776,7 +23704,7 @@
         <x:v>mobile_terminal_soul_sections_1_title</x:v>
       </x:c>
       <x:c r="C144" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D144" t="str">
         <x:v>5031</x:v>
@@ -22890,7 +23818,7 @@
         <x:v>mobile_terminal_soul_sections_1_meta</x:v>
       </x:c>
       <x:c r="C145" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D145" t="str">
         <x:v>5032</x:v>
@@ -23004,7 +23932,7 @@
         <x:v>mobile_terminal_soul_sections_1_summary</x:v>
       </x:c>
       <x:c r="C146" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D146" t="str">
         <x:v>5033</x:v>
@@ -23118,7 +24046,7 @@
         <x:v>mobile_terminal_soul_sections_1_details_0</x:v>
       </x:c>
       <x:c r="C147" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D147" t="str">
         <x:v>5034</x:v>
@@ -23232,7 +24160,7 @@
         <x:v>mobile_terminal_soul_sections_1_details_1</x:v>
       </x:c>
       <x:c r="C148" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D148" t="str">
         <x:v>5035</x:v>
@@ -23346,7 +24274,7 @@
         <x:v>mobile_terminal_soul_sections_2_title</x:v>
       </x:c>
       <x:c r="C149" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D149" t="str">
         <x:v>5036</x:v>
@@ -23460,7 +24388,7 @@
         <x:v>mobile_terminal_soul_sections_2_meta</x:v>
       </x:c>
       <x:c r="C150" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D150" t="str">
         <x:v>5037</x:v>
@@ -23574,7 +24502,7 @@
         <x:v>mobile_terminal_soul_sections_2_summary</x:v>
       </x:c>
       <x:c r="C151" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D151" t="str">
         <x:v>5038</x:v>
@@ -23688,7 +24616,7 @@
         <x:v>mobile_terminal_soul_sections_2_details_0</x:v>
       </x:c>
       <x:c r="C152" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D152" t="str">
         <x:v>5039</x:v>
@@ -23802,7 +24730,7 @@
         <x:v>mobile_terminal_soul_sections_2_details_1</x:v>
       </x:c>
       <x:c r="C153" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D153" t="str">
         <x:v>5040</x:v>
@@ -23916,7 +24844,7 @@
         <x:v>mobile_terminal_soul_sections_3_title</x:v>
       </x:c>
       <x:c r="C154" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D154" t="str">
         <x:v>5041</x:v>
@@ -24030,7 +24958,7 @@
         <x:v>mobile_terminal_soul_sections_3_meta</x:v>
       </x:c>
       <x:c r="C155" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D155" t="str">
         <x:v>5042</x:v>
@@ -24144,7 +25072,7 @@
         <x:v>mobile_terminal_soul_sections_3_summary</x:v>
       </x:c>
       <x:c r="C156" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D156" t="str">
         <x:v>5043</x:v>
@@ -24258,7 +25186,7 @@
         <x:v>mobile_terminal_soul_sections_3_details_0</x:v>
       </x:c>
       <x:c r="C157" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D157" t="str">
         <x:v>5044</x:v>
@@ -24372,7 +25300,7 @@
         <x:v>mobile_terminal_soul_sections_3_details_1</x:v>
       </x:c>
       <x:c r="C158" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D158" t="str">
         <x:v>5045</x:v>
@@ -24600,7 +25528,7 @@
         <x:v>mobile_terminal_contact_name</x:v>
       </x:c>
       <x:c r="C160" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D160" t="str">
         <x:v>5047</x:v>
@@ -24714,7 +25642,7 @@
         <x:v>mobile_terminal_contact_roleLine</x:v>
       </x:c>
       <x:c r="C161" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D161" t="str">
         <x:v>5048</x:v>
@@ -24828,7 +25756,7 @@
         <x:v>mobile_terminal_contact_lines_0_label</x:v>
       </x:c>
       <x:c r="C162" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D162" t="str">
         <x:v>5049</x:v>
@@ -24942,7 +25870,7 @@
         <x:v>mobile_terminal_contact_lines_0_values_0_text</x:v>
       </x:c>
       <x:c r="C163" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D163" t="str">
         <x:v>5050</x:v>
@@ -25056,7 +25984,7 @@
         <x:v>mobile_terminal_contact_lines_0_values_0_href</x:v>
       </x:c>
       <x:c r="C164" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D164" t="str">
         <x:v>5051</x:v>
@@ -25170,7 +26098,7 @@
         <x:v>mobile_terminal_contact_lines_0_values_1_text</x:v>
       </x:c>
       <x:c r="C165" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D165" t="str">
         <x:v>5052</x:v>
@@ -25284,7 +26212,7 @@
         <x:v>mobile_terminal_contact_lines_0_values_1_href</x:v>
       </x:c>
       <x:c r="C166" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D166" t="str">
         <x:v>5053</x:v>
@@ -25398,7 +26326,7 @@
         <x:v>mobile_terminal_contact_lines_1_label</x:v>
       </x:c>
       <x:c r="C167" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D167" t="str">
         <x:v>5054</x:v>
@@ -25512,7 +26440,7 @@
         <x:v>mobile_terminal_contact_lines_1_values_0_text</x:v>
       </x:c>
       <x:c r="C168" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D168" t="str">
         <x:v>5055</x:v>
@@ -25626,7 +26554,7 @@
         <x:v>mobile_terminal_contact_lines_2_label</x:v>
       </x:c>
       <x:c r="C169" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D169" t="str">
         <x:v>5056</x:v>
@@ -25740,7 +26668,7 @@
         <x:v>mobile_terminal_contact_lines_2_values_0_text</x:v>
       </x:c>
       <x:c r="C170" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D170" t="str">
         <x:v>5057</x:v>
@@ -25854,7 +26782,7 @@
         <x:v>mobile_terminal_contact_lines_2_values_0_href</x:v>
       </x:c>
       <x:c r="C171" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D171" t="str">
         <x:v>5058</x:v>
@@ -25968,7 +26896,7 @@
         <x:v>mobile_terminal_contact_lines_3_label</x:v>
       </x:c>
       <x:c r="C172" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D172" t="str">
         <x:v>5059</x:v>
@@ -26082,7 +27010,7 @@
         <x:v>mobile_terminal_contact_lines_3_values_0_text</x:v>
       </x:c>
       <x:c r="C173" t="str">
-        <x:v>Y</x:v>
+        <x:v>N</x:v>
       </x:c>
       <x:c r="D173" t="str">
         <x:v>5060</x:v>
@@ -28111,10 +29039,10 @@
         <x:v>profile.overviewSignal.0</x:v>
       </x:c>
       <x:c r="CH190" t="str">
-        <x:v>Architecture + creative technology practice between New York and Shanghai.</x:v>
+        <x:v>Architectural design and AI visual practice based in Shenzhen.</x:v>
       </x:c>
       <x:c r="CI190" t="str">
-        <x:v>位于 New York / Shanghai 之间的建筑 + creative technology 实践。</x:v>
+        <x:v>现居深圳，从事建筑设计与 AI 视觉创作。</x:v>
       </x:c>
       <x:c r="CJ190" t="str"/>
       <x:c r="CK190" t="str"/>

</xml_diff>